<commit_message>
Update agent metadata and document phase 1 baseline reviews
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
+++ b/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
@@ -13,15 +13,17 @@
     <sheet name="Completeness" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Progress" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Tracking guide" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Baseline audit" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Threat Map'!$A$5:$M$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Completeness'!$A$1:$N$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Completeness'!$A$1:$N$114</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Completeness'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Progress'!$A$1:$D$27</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Progress'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tracking guide'!$A$1:$B$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Tracking guide'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Baseline audit'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -388,7 +390,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Phase1Tracker" displayName="Phase1Tracker" ref="A1:N105" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Phase1Tracker" displayName="Phase1Tracker" ref="A1:N114" headerRowCount="1">
   <autoFilter ref="A1:N105"/>
   <tableColumns count="14">
     <tableColumn id="1" name="ID"/>
@@ -405,6 +407,21 @@
     <tableColumn id="12" name="Reviewed date"/>
     <tableColumn id="13" name="Evidence / result link"/>
     <tableColumn id="14" name="Due date"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BaselineAudit" displayName="BaselineAudit" ref="A1:F10" headerRowCount="1">
+  <autoFilter ref="A1:F10"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="Area"/>
+    <tableColumn id="3" name="Classification / confidence"/>
+    <tableColumn id="4" name="Observation"/>
+    <tableColumn id="5" name="Next action"/>
+    <tableColumn id="6" name="Related requirements"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -1877,7 +1894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N105"/>
+  <dimension ref="A1:N114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" style="14" min="1" max="1"/>
@@ -3185,7 +3202,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M21" s="28" t="n"/>
+      <c r="M21" s="28" t="inlineStr">
+        <is>
+          <t>BASE-05: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N21" s="28" t="n"/>
     </row>
     <row r="22" ht="90" customHeight="1" s="14">
@@ -3441,7 +3462,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M25" s="28" t="n"/>
+      <c r="M25" s="28" t="inlineStr">
+        <is>
+          <t>BASE-05: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N25" s="28" t="n"/>
     </row>
     <row r="26" ht="90" customHeight="1" s="14">
@@ -3505,7 +3530,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M26" s="28" t="n"/>
+      <c r="M26" s="28" t="inlineStr">
+        <is>
+          <t>BASE-04: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N26" s="28" t="n"/>
     </row>
     <row r="27" ht="90" customHeight="1" s="14">
@@ -3569,7 +3598,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M27" s="28" t="n"/>
+      <c r="M27" s="28" t="inlineStr">
+        <is>
+          <t>BASE-04: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N27" s="28" t="n"/>
     </row>
     <row r="28" ht="90" customHeight="1" s="14">
@@ -3633,7 +3666,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M28" s="28" t="n"/>
+      <c r="M28" s="28" t="inlineStr">
+        <is>
+          <t>BASE-04: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N28" s="28" t="n"/>
     </row>
     <row r="29" ht="90" customHeight="1" s="14">
@@ -4017,7 +4054,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M34" s="28" t="n"/>
+      <c r="M34" s="28" t="inlineStr">
+        <is>
+          <t>BASE-05: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N34" s="28" t="n"/>
     </row>
     <row r="35" ht="90" customHeight="1" s="14">
@@ -4081,7 +4122,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M35" s="28" t="n"/>
+      <c r="M35" s="28" t="inlineStr">
+        <is>
+          <t>BASE-06: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N35" s="28" t="n"/>
     </row>
     <row r="36" ht="90" customHeight="1" s="14">
@@ -4145,7 +4190,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M36" s="28" t="n"/>
+      <c r="M36" s="28" t="inlineStr">
+        <is>
+          <t>BASE-06: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N36" s="28" t="n"/>
     </row>
     <row r="37" ht="90" customHeight="1" s="14">
@@ -5077,7 +5126,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M51" s="28" t="n"/>
+      <c r="M51" s="28" t="inlineStr">
+        <is>
+          <t>BASE-09: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N51" s="28" t="n"/>
     </row>
     <row r="52" ht="90" customHeight="1" s="14">
@@ -6273,7 +6326,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M70" s="28" t="n"/>
+      <c r="M70" s="28" t="inlineStr">
+        <is>
+          <t>BASE-02: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N70" s="28" t="n"/>
     </row>
     <row r="71" ht="90" customHeight="1" s="14">
@@ -6453,7 +6510,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M73" s="28" t="n"/>
+      <c r="M73" s="28" t="inlineStr">
+        <is>
+          <t>BASE-08: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N73" s="28" t="n"/>
     </row>
     <row r="74" ht="90" customHeight="1" s="14">
@@ -7001,7 +7062,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M82" s="28" t="n"/>
+      <c r="M82" s="28" t="inlineStr">
+        <is>
+          <t>BASE-03: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N82" s="28" t="n"/>
     </row>
     <row r="83" ht="90" customHeight="1" s="14">
@@ -7245,7 +7310,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M86" s="28" t="n"/>
+      <c r="M86" s="28" t="inlineStr">
+        <is>
+          <t>BASE-01: docs/reviews/phase1-baseline/README.md; BASE-03: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N86" s="28" t="n"/>
     </row>
     <row r="87" ht="90" customHeight="1" s="14">
@@ -7305,7 +7374,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M87" s="28" t="n"/>
+      <c r="M87" s="28" t="inlineStr">
+        <is>
+          <t>BASE-05: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N87" s="28" t="n"/>
     </row>
     <row r="88" ht="90" customHeight="1" s="14">
@@ -7365,7 +7438,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M88" s="28" t="n"/>
+      <c r="M88" s="28" t="inlineStr">
+        <is>
+          <t>BASE-04: docs/reviews/phase1-baseline/README.md; BASE-05: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N88" s="28" t="n"/>
     </row>
     <row r="89" ht="90" customHeight="1" s="14">
@@ -7485,7 +7562,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M90" s="28" t="n"/>
+      <c r="M90" s="28" t="inlineStr">
+        <is>
+          <t>BASE-07: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N90" s="28" t="n"/>
     </row>
     <row r="91" ht="90" customHeight="1" s="14">
@@ -7545,7 +7626,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M91" s="28" t="n"/>
+      <c r="M91" s="28" t="inlineStr">
+        <is>
+          <t>BASE-06: docs/reviews/phase1-baseline/README.md; BASE-09: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N91" s="28" t="n"/>
     </row>
     <row r="92" ht="90" customHeight="1" s="14">
@@ -7609,7 +7694,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M92" s="28" t="n"/>
+      <c r="M92" s="28" t="inlineStr">
+        <is>
+          <t>BASE-09: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N92" s="28" t="n"/>
     </row>
     <row r="93" ht="90" customHeight="1" s="14">
@@ -7669,7 +7758,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M93" s="28" t="n"/>
+      <c r="M93" s="28" t="inlineStr">
+        <is>
+          <t>BASE-01: docs/reviews/phase1-baseline/README.md; BASE-03: docs/reviews/phase1-baseline/README.md; BASE-08: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N93" s="28" t="n"/>
     </row>
     <row r="94" ht="90" customHeight="1" s="14">
@@ -7969,7 +8062,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M98" s="28" t="n"/>
+      <c r="M98" s="28" t="inlineStr">
+        <is>
+          <t>BASE-02: docs/reviews/phase1-baseline/README.md; BASE-07: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N98" s="28" t="n"/>
     </row>
     <row r="99" ht="90" customHeight="1" s="14">
@@ -8029,7 +8126,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M99" s="28" t="n"/>
+      <c r="M99" s="28" t="inlineStr">
+        <is>
+          <t>BASE-02: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N99" s="28" t="n"/>
     </row>
     <row r="100" ht="90" customHeight="1" s="14">
@@ -8089,7 +8190,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M100" s="28" t="n"/>
+      <c r="M100" s="28" t="inlineStr">
+        <is>
+          <t>BASE-02: docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
       <c r="N100" s="28" t="n"/>
     </row>
     <row r="101" ht="90" customHeight="1" s="14">
@@ -8400,8 +8505,620 @@
       <c r="M105" s="28" t="n"/>
       <c r="N105" s="28" t="n"/>
     </row>
+    <row r="106" ht="100" customHeight="1" s="14">
+      <c r="A106" s="28" t="inlineStr">
+        <is>
+          <t>BASE-01</t>
+        </is>
+      </c>
+      <c r="B106" s="28" t="inlineStr">
+        <is>
+          <t>Baseline audit</t>
+        </is>
+      </c>
+      <c r="C106" s="28" t="inlineStr">
+        <is>
+          <t>Assembler/compiler</t>
+        </is>
+      </c>
+      <c r="D106" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1 assurance</t>
+        </is>
+      </c>
+      <c r="E106" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F106" s="28" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G106" s="28" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="H106" s="28" t="inlineStr">
+        <is>
+          <t>SIM-01; REL-03</t>
+        </is>
+      </c>
+      <c r="I106" s="28" t="inlineStr">
+        <is>
+          <t>Confirmed dependency-initialization failure; not an ISA verdict. Existing assembler workflow throws TypeError: ChurchAssembler is not a constructor at compiler line 220. Fresh in-memory probe reproduces it with global assembler undefined; injecting the real constructor removes this exception (the sample still has one compile diagnostic).</t>
+        </is>
+      </c>
+      <c r="J106" s="28" t="inlineStr">
+        <is>
+          <t>Establish explicit Node/compiler dependency setup and regression coverage; rerun isolated assembler suite before interpreting encoding failures. Do not weaken retired-opcode diagnostics.</t>
+        </is>
+      </c>
+      <c r="K106" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="L106" s="28" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="M106" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="N106" s="28" t="n"/>
+    </row>
+    <row r="107" ht="100" customHeight="1" s="14">
+      <c r="A107" s="28" t="inlineStr">
+        <is>
+          <t>BASE-02</t>
+        </is>
+      </c>
+      <c r="B107" s="28" t="inlineStr">
+        <is>
+          <t>Baseline audit</t>
+        </is>
+      </c>
+      <c r="C107" s="28" t="inlineStr">
+        <is>
+          <t>Selected resident identity</t>
+        </is>
+      </c>
+      <c r="D107" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1 assurance</t>
+        </is>
+      </c>
+      <c r="E107" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F107" s="28" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G107" s="28" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="H107" s="28" t="inlineStr">
+        <is>
+          <t>RES-SelfTest; RES-WukongCallHome; RES-CapabilityTest; IDE-03</t>
+        </is>
+      </c>
+      <c r="I107" s="28" t="inlineStr">
+        <is>
+          <t>Confirmed saved-configuration/catalog mismatch. Selected SelfTest has one active matching row; selected WukongCallHome and CapabilityTest have zero. All three selected binary hashes match their files. One existing LUMP-consistency test reports this class of failure.</t>
+        </is>
+      </c>
+      <c r="J107" s="28" t="inlineStr">
+        <is>
+          <t>Review exact selected artifact versus intended revision and manifest history; propose an explicit approved reconciliation. Do not silently select latest, rewrite history or regenerate images.</t>
+        </is>
+      </c>
+      <c r="K107" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="L107" s="28" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="M107" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="N107" s="28" t="n"/>
+    </row>
+    <row r="108" ht="100" customHeight="1" s="14">
+      <c r="A108" s="28" t="inlineStr">
+        <is>
+          <t>BASE-03</t>
+        </is>
+      </c>
+      <c r="B108" s="28" t="inlineStr">
+        <is>
+          <t>Baseline audit</t>
+        </is>
+      </c>
+      <c r="C108" s="28" t="inlineStr">
+        <is>
+          <t>LUMP GT validator</t>
+        </is>
+      </c>
+      <c r="D108" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1 assurance</t>
+        </is>
+      </c>
+      <c r="E108" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F108" s="28" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G108" s="28" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="H108" s="28" t="inlineStr">
+        <is>
+          <t>SIM-01; SEAL-02; REL-03</t>
+        </is>
+      </c>
+      <c r="I108" s="28" t="inlineStr">
+        <is>
+          <t>Legacy-oracle conflict; affected binary validity not established. Four reported R22 failures use _gt_word0_violation, which declares bit 26 spare and rejects it. The test itself notes Abstract GT encodings use bits 26:25=11. The four reported cases are 04b2913d, 3b057bbb, Ethernet.1.b169bba4 and Ethernet.1.fc72b0e3.</t>
+        </is>
+      </c>
+      <c r="J108" s="28" t="inlineStr">
+        <is>
+          <t>Classify each rejected word by approved type and permissions; replace the obsolete blanket rule only under the current contract. Do not declare all four artifacts valid just because the old rule is wrong.</t>
+        </is>
+      </c>
+      <c r="K108" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="L108" s="28" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="M108" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="N108" s="28" t="n"/>
+    </row>
+    <row r="109" ht="100" customHeight="1" s="14">
+      <c r="A109" s="28" t="inlineStr">
+        <is>
+          <t>BASE-04</t>
+        </is>
+      </c>
+      <c r="B109" s="28" t="inlineStr">
+        <is>
+          <t>Baseline audit</t>
+        </is>
+      </c>
+      <c r="C109" s="28" t="inlineStr">
+        <is>
+          <t>Boot-image agreement</t>
+        </is>
+      </c>
+      <c r="D109" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1 assurance</t>
+        </is>
+      </c>
+      <c r="E109" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F109" s="28" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G109" s="28" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="H109" s="28" t="inlineStr">
+        <is>
+          <t>SIM-03; H10; H11; H12</t>
+        </is>
+      </c>
+      <c r="I109" s="28" t="inlineStr">
+        <is>
+          <t>Shared generator/fixture contract failure; root cause provisional. All 18 reported failures stop at mandatory NS slot 2 is zeroed; 8 other cases passed. Tests build synthetic Boot.Abstr fixtures in temporary directories; generator still requires legacy slots (0,1,2,3,4,5,6,10). Agreement is not reached in these failed cases.</t>
+        </is>
+      </c>
+      <c r="J109" s="28" t="inlineStr">
+        <is>
+          <t>Trace fixture selection, generation policy and validator mode in an isolated copy. Reconcile approved slot-2 entry versus legacy device/profile semantics; do not remove validation merely to pass tests.</t>
+        </is>
+      </c>
+      <c r="K109" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="L109" s="28" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="M109" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="N109" s="28" t="n"/>
+    </row>
+    <row r="110" ht="100" customHeight="1" s="14">
+      <c r="A110" s="28" t="inlineStr">
+        <is>
+          <t>BASE-05</t>
+        </is>
+      </c>
+      <c r="B110" s="28" t="inlineStr">
+        <is>
+          <t>Baseline audit</t>
+        </is>
+      </c>
+      <c r="C110" s="28" t="inlineStr">
+        <is>
+          <t>RTL boot/control</t>
+        </is>
+      </c>
+      <c r="D110" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1 assurance</t>
+        </is>
+      </c>
+      <c r="E110" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F110" s="28" t="inlineStr">
+        <is>
+          <t>Needs verification</t>
+        </is>
+      </c>
+      <c r="G110" s="28" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="H110" s="28" t="inlineStr">
+        <is>
+          <t>SIM-02; SIM-03; H05; H09; H18</t>
+        </is>
+      </c>
+      <c r="I110" s="28" t="inlineStr">
+        <is>
+          <t>Unresolved fixture/implementation/oracle failures. Existing run: 8 failed, 46 passed. Failures cover SWITCH outcomes, delayed-fault issuer attribution, nested CALL/RETURN and saved-PC validation. No fresh RTL simulation was performed.</t>
+        </is>
+      </c>
+      <c r="J110" s="28" t="inlineStr">
+        <is>
+          <t>Capture instruction words and pre-fault state, verify approved fixture encodings, then replay minimal isolated cases. Keep implementation defects possible until evidence excludes them.</t>
+        </is>
+      </c>
+      <c r="K110" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="L110" s="28" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="M110" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="N110" s="28" t="n"/>
+    </row>
+    <row r="111" ht="100" customHeight="1" s="14">
+      <c r="A111" s="28" t="inlineStr">
+        <is>
+          <t>BASE-06</t>
+        </is>
+      </c>
+      <c r="B111" s="28" t="inlineStr">
+        <is>
+          <t>Baseline audit</t>
+        </is>
+      </c>
+      <c r="C111" s="28" t="inlineStr">
+        <is>
+          <t>Generated initialization</t>
+        </is>
+      </c>
+      <c r="D111" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1 assurance</t>
+        </is>
+      </c>
+      <c r="E111" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F111" s="28" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G111" s="28" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="H111" s="28" t="inlineStr">
+        <is>
+          <t>REL-01; H19; H20</t>
+        </is>
+      </c>
+      <c r="I111" s="28" t="inlineStr">
+        <is>
+          <t>Reported generated-artifact/source mismatch; not freshly recomputed. Existing guard: RTLIL init ROM 2693 entries versus Python source 2694; 1 failed, 25 passed in that suite.</t>
+        </is>
+      </c>
+      <c r="J111" s="28" t="inlineStr">
+        <is>
+          <t>Freeze source and approved image first; then regenerate and qualify exact outputs under separate authorization. Do not equate a one-entry count fix with a qualified bitstream.</t>
+        </is>
+      </c>
+      <c r="K111" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="L111" s="28" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="M111" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="N111" s="28" t="n"/>
+    </row>
+    <row r="112" ht="100" customHeight="1" s="14">
+      <c r="A112" s="28" t="inlineStr">
+        <is>
+          <t>BASE-07</t>
+        </is>
+      </c>
+      <c r="B112" s="28" t="inlineStr">
+        <is>
+          <t>Baseline audit</t>
+        </is>
+      </c>
+      <c r="C112" s="28" t="inlineStr">
+        <is>
+          <t>SelfTest freshness</t>
+        </is>
+      </c>
+      <c r="D112" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1 assurance</t>
+        </is>
+      </c>
+      <c r="E112" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F112" s="28" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G112" s="28" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="H112" s="28" t="inlineStr">
+        <is>
+          <t>RES-SelfTest; SIM-05</t>
+        </is>
+      </c>
+      <c r="I112" s="28" t="inlineStr">
+        <is>
+          <t>Reported source/entry-format drift, not observed execution failure. Selected SelfTest hash is intact. Existing freshness guard says instruction body MATCH, embedded text DIFFERENT, method-entry format DIFFERENT. The first failing command prevents the chained guard-test command from running.</t>
+        </is>
+      </c>
+      <c r="J112" s="28" t="inlineStr">
+        <is>
+          <t>Independently inspect actual CALL dispatch/decoder behavior for the exact selected artifact before proposing replacement. Preserve the selected bytes and distinguish source freshness from execution compatibility.</t>
+        </is>
+      </c>
+      <c r="K112" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="L112" s="28" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="M112" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="N112" s="28" t="n"/>
+    </row>
+    <row r="113" ht="100" customHeight="1" s="14">
+      <c r="A113" s="28" t="inlineStr">
+        <is>
+          <t>BASE-08</t>
+        </is>
+      </c>
+      <c r="B113" s="28" t="inlineStr">
+        <is>
+          <t>Baseline audit</t>
+        </is>
+      </c>
+      <c r="C113" s="28" t="inlineStr">
+        <is>
+          <t>API reference suite</t>
+        </is>
+      </c>
+      <c r="D113" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1 assurance</t>
+        </is>
+      </c>
+      <c r="E113" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F113" s="28" t="inlineStr">
+        <is>
+          <t>Needs verification</t>
+        </is>
+      </c>
+      <c r="G113" s="28" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="H113" s="28" t="inlineStr">
+        <is>
+          <t>IDE-06; REL-03</t>
+        </is>
+      </c>
+      <c r="I113" s="28" t="inlineStr">
+        <is>
+          <t>Probable fixture/contract drift; not a fresh test result. Existing run fails in test_abs_saved_api.js: compiled method declarations unavailable. The fixture invokes _formatLumpApiDefinition('LED', []); failure occurs before the advertised reference comparison completes.</t>
+        </is>
+      </c>
+      <c r="J113" s="28" t="inlineStr">
+        <is>
+          <t>Supply authentic compiled metadata in the fixture, or establish why valid metadata is lost; retain fail-closed refusal to infer API from another LUMP.</t>
+        </is>
+      </c>
+      <c r="K113" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="L113" s="28" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="M113" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="N113" s="28" t="n"/>
+    </row>
+    <row r="114" ht="100" customHeight="1" s="14">
+      <c r="A114" s="28" t="inlineStr">
+        <is>
+          <t>BASE-09</t>
+        </is>
+      </c>
+      <c r="B114" s="28" t="inlineStr">
+        <is>
+          <t>Baseline audit</t>
+        </is>
+      </c>
+      <c r="C114" s="28" t="inlineStr">
+        <is>
+          <t>Bitstream provenance</t>
+        </is>
+      </c>
+      <c r="D114" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1 assurance</t>
+        </is>
+      </c>
+      <c r="E114" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F114" s="28" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G114" s="28" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="H114" s="28" t="inlineStr">
+        <is>
+          <t>REL-01; REL-02; CM-H</t>
+        </is>
+      </c>
+      <c r="I114" s="28" t="inlineStr">
+        <is>
+          <t>Confirmed current-source drift from recorded build. Fresh hash comparison finds 22 of 39 recorded input fingerprints differ from current files. The record's historical “verified” label is not qualification of today's source.</t>
+        </is>
+      </c>
+      <c r="J114" s="28" t="inlineStr">
+        <is>
+          <t>Freeze the candidate source/configuration; obtain matching generation, build/timing, artifact hashes and authorized physical evidence. Do not relabel the historical bitstream.</t>
+        </is>
+      </c>
+      <c r="K114" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="L114" s="28" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="M114" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/README.md</t>
+        </is>
+      </c>
+      <c r="N114" s="28" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N105"/>
+  <autoFilter ref="A1:N114"/>
   <conditionalFormatting sqref="F2:F10000">
     <cfRule type="expression" priority="1" dxfId="4">
       <formula>F2="Complete"</formula>
@@ -8438,7 +9155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" style="14" min="1" max="1"/>
@@ -8885,6 +9602,25 @@
       </c>
       <c r="D27" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A27,Completeness!F2:F10000,"Blocked")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="28" t="inlineStr">
+        <is>
+          <t>Baseline audit</t>
+        </is>
+      </c>
+      <c r="B28" s="28">
+        <f>COUNTIF(Completeness!B2:B10000,A28)</f>
+        <v/>
+      </c>
+      <c r="C28" s="28">
+        <f>COUNTIFS(Completeness!B2:B10000,A28,Completeness!F2:F10000,"Complete")</f>
+        <v/>
+      </c>
+      <c r="D28" s="28">
+        <f>COUNTIFS(Completeness!B2:B10000,A28,Completeness!F2:F10000,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -8901,7 +9637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" style="14" min="1" max="1"/>
@@ -9066,9 +9802,367 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Baseline audit</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Nine root-cause groups. Workflow results are existing observations, not fresh reruns. Only the compiler dependency and read-only hash/binding probes were reproduced. See repository audit report.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="14" min="1" max="1"/>
+    <col width="26" customWidth="1" style="14" min="2" max="2"/>
+    <col width="55" customWidth="1" style="14" min="3" max="3"/>
+    <col width="95" customWidth="1" style="14" min="4" max="4"/>
+    <col width="90" customWidth="1" style="14" min="5" max="5"/>
+    <col width="55" customWidth="1" style="14" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="27" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C1" s="27" t="inlineStr">
+        <is>
+          <t>Classification / confidence</t>
+        </is>
+      </c>
+      <c r="D1" s="27" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="E1" s="27" t="inlineStr">
+        <is>
+          <t>Next action</t>
+        </is>
+      </c>
+      <c r="F1" s="27" t="inlineStr">
+        <is>
+          <t>Related requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="110" customHeight="1" s="14">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>BASE-01</t>
+        </is>
+      </c>
+      <c r="B2" s="28" t="inlineStr">
+        <is>
+          <t>Assembler/compiler</t>
+        </is>
+      </c>
+      <c r="C2" s="28" t="inlineStr">
+        <is>
+          <t>Confirmed dependency-initialization failure; not an ISA verdict</t>
+        </is>
+      </c>
+      <c r="D2" s="28" t="inlineStr">
+        <is>
+          <t>Existing assembler workflow throws TypeError: ChurchAssembler is not a constructor at compiler line 220. Fresh in-memory probe reproduces it with global assembler undefined; injecting the real constructor removes this exception (the sample still has one compile diagnostic).</t>
+        </is>
+      </c>
+      <c r="E2" s="28" t="inlineStr">
+        <is>
+          <t>Establish explicit Node/compiler dependency setup and regression coverage; rerun isolated assembler suite before interpreting encoding failures. Do not weaken retired-opcode diagnostics.</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>SIM-01; REL-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="110" customHeight="1" s="14">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>BASE-02</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>Selected resident identity</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>Confirmed saved-configuration/catalog mismatch</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>Selected SelfTest has one active matching row; selected WukongCallHome and CapabilityTest have zero. All three selected binary hashes match their files. One existing LUMP-consistency test reports this class of failure.</t>
+        </is>
+      </c>
+      <c r="E3" s="28" t="inlineStr">
+        <is>
+          <t>Review exact selected artifact versus intended revision and manifest history; propose an explicit approved reconciliation. Do not silently select latest, rewrite history or regenerate images.</t>
+        </is>
+      </c>
+      <c r="F3" s="28" t="inlineStr">
+        <is>
+          <t>RES-SelfTest; RES-WukongCallHome; RES-CapabilityTest; IDE-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="110" customHeight="1" s="14">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>BASE-03</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>LUMP GT validator</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>Legacy-oracle conflict; affected binary validity not established</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Four reported R22 failures use _gt_word0_violation, which declares bit 26 spare and rejects it. The test itself notes Abstract GT encodings use bits 26:25=11. The four reported cases are 04b2913d, 3b057bbb, Ethernet.1.b169bba4 and Ethernet.1.fc72b0e3.</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>Classify each rejected word by approved type and permissions; replace the obsolete blanket rule only under the current contract. Do not declare all four artifacts valid just because the old rule is wrong.</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>SIM-01; SEAL-02; REL-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="110" customHeight="1" s="14">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>BASE-04</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>Boot-image agreement</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>Shared generator/fixture contract failure; root cause provisional</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>All 18 reported failures stop at mandatory NS slot 2 is zeroed; 8 other cases passed. Tests build synthetic Boot.Abstr fixtures in temporary directories; generator still requires legacy slots (0,1,2,3,4,5,6,10). Agreement is not reached in these failed cases.</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="inlineStr">
+        <is>
+          <t>Trace fixture selection, generation policy and validator mode in an isolated copy. Reconcile approved slot-2 entry versus legacy device/profile semantics; do not remove validation merely to pass tests.</t>
+        </is>
+      </c>
+      <c r="F5" s="28" t="inlineStr">
+        <is>
+          <t>SIM-03; H10; H11; H12</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="110" customHeight="1" s="14">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>BASE-05</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>RTL boot/control</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>Unresolved fixture/implementation/oracle failures</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>Existing run: 8 failed, 46 passed. Failures cover SWITCH outcomes, delayed-fault issuer attribution, nested CALL/RETURN and saved-PC validation. No fresh RTL simulation was performed.</t>
+        </is>
+      </c>
+      <c r="E6" s="28" t="inlineStr">
+        <is>
+          <t>Capture instruction words and pre-fault state, verify approved fixture encodings, then replay minimal isolated cases. Keep implementation defects possible until evidence excludes them.</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>SIM-02; SIM-03; H05; H09; H18</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="110" customHeight="1" s="14">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>BASE-06</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>Generated initialization</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr">
+        <is>
+          <t>Reported generated-artifact/source mismatch; not freshly recomputed</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>Existing guard: RTLIL init ROM 2693 entries versus Python source 2694; 1 failed, 25 passed in that suite.</t>
+        </is>
+      </c>
+      <c r="E7" s="28" t="inlineStr">
+        <is>
+          <t>Freeze source and approved image first; then regenerate and qualify exact outputs under separate authorization. Do not equate a one-entry count fix with a qualified bitstream.</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>REL-01; H19; H20</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="110" customHeight="1" s="14">
+      <c r="A8" s="28" t="inlineStr">
+        <is>
+          <t>BASE-07</t>
+        </is>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>SelfTest freshness</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>Reported source/entry-format drift, not observed execution failure</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="inlineStr">
+        <is>
+          <t>Selected SelfTest hash is intact. Existing freshness guard says instruction body MATCH, embedded text DIFFERENT, method-entry format DIFFERENT. The first failing command prevents the chained guard-test command from running.</t>
+        </is>
+      </c>
+      <c r="E8" s="28" t="inlineStr">
+        <is>
+          <t>Independently inspect actual CALL dispatch/decoder behavior for the exact selected artifact before proposing replacement. Preserve the selected bytes and distinguish source freshness from execution compatibility.</t>
+        </is>
+      </c>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>RES-SelfTest; SIM-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="110" customHeight="1" s="14">
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>BASE-08</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>API reference suite</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="inlineStr">
+        <is>
+          <t>Probable fixture/contract drift; not a fresh test result</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="inlineStr">
+        <is>
+          <t>Existing run fails in test_abs_saved_api.js: compiled method declarations unavailable. The fixture invokes _formatLumpApiDefinition('LED', []); failure occurs before the advertised reference comparison completes.</t>
+        </is>
+      </c>
+      <c r="E9" s="28" t="inlineStr">
+        <is>
+          <t>Supply authentic compiled metadata in the fixture, or establish why valid metadata is lost; retain fail-closed refusal to infer API from another LUMP.</t>
+        </is>
+      </c>
+      <c r="F9" s="28" t="inlineStr">
+        <is>
+          <t>IDE-06; REL-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="110" customHeight="1" s="14">
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>BASE-09</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>Bitstream provenance</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="inlineStr">
+        <is>
+          <t>Confirmed current-source drift from recorded build</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>Fresh hash comparison finds 22 of 39 recorded input fingerprints differ from current files. The record's historical “verified” label is not qualification of today's source.</t>
+        </is>
+      </c>
+      <c r="E10" s="28" t="inlineStr">
+        <is>
+          <t>Freeze the candidate source/configuration; obtain matching generation, build/timing, artifact hashes and authorized physical evidence. Do not relabel the historical bitstream.</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="inlineStr">
+        <is>
+          <t>REL-01; REL-02; CM-H</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update agent metadata and documentation for phase one threat testing
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
+++ b/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
@@ -8586,7 +8586,7 @@
       </c>
       <c r="C107" s="28" t="inlineStr">
         <is>
-          <t>Selected resident identity</t>
+          <t>Namespace authority</t>
         </is>
       </c>
       <c r="D107" s="28" t="inlineStr">
@@ -8616,12 +8616,12 @@
       </c>
       <c r="I107" s="28" t="inlineStr">
         <is>
-          <t>Confirmed saved-configuration/catalog mismatch. Selected SelfTest has one active matching row; selected WukongCallHome and CapabilityTest have zero. All three selected binary hashes match their files. One existing LUMP-consistency test reports this class of failure.</t>
+          <t>Test imposes a competing manifest-authority requirement. Selected SelfTest has one active matching catalog row; selected WukongCallHome and CapabilityTest have zero. All three selected binary hashes match their files. Genesis confirms the approved Namespace list is authoritative; missing active catalog rows do not invalidate these selections. Hash agreement alone is not full execution qualification.</t>
         </is>
       </c>
       <c r="J107" s="28" t="inlineStr">
         <is>
-          <t>Review exact selected artifact versus intended revision and manifest history; propose an explicit approved reconciliation. Do not silently select latest, rewrite history or regenerate images.</t>
+          <t>Correct the test's requirement for an active manifest row and inspect consumers for equivalent catalog vetoes. Validate exact Namespace-selected bytes, identity, permissions, allocation and binding directly. A library/history index may locate files but cannot override approval. No catalog repair or reselection is required merely to satisfy this test.</t>
         </is>
       </c>
       <c r="K107" s="28" t="inlineStr">
@@ -9637,7 +9637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" style="14" min="1" max="1"/>
@@ -9803,14 +9803,26 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Baseline audit</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>Nine root-cause groups. Workflow results are existing observations, not fresh reruns. Only the compiler dependency and read-only hash/binding probes were reproduced. See repository audit report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="80" customHeight="1" s="14">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Namespace authority</t>
+        </is>
+      </c>
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>Genesis-approved Namespace selection is authoritative. A manifest may index library/history files, but missing, archived or duplicate catalog rows cannot veto independently verified selected bytes. BASE-02 tracks the competing test requirement, not a request to repair approved selections.</t>
         </is>
       </c>
     </row>
@@ -9910,22 +9922,22 @@
       </c>
       <c r="B3" s="28" t="inlineStr">
         <is>
-          <t>Selected resident identity</t>
+          <t>Namespace authority</t>
         </is>
       </c>
       <c r="C3" s="28" t="inlineStr">
         <is>
-          <t>Confirmed saved-configuration/catalog mismatch</t>
+          <t>Test imposes a competing manifest-authority requirement</t>
         </is>
       </c>
       <c r="D3" s="28" t="inlineStr">
         <is>
-          <t>Selected SelfTest has one active matching row; selected WukongCallHome and CapabilityTest have zero. All three selected binary hashes match their files. One existing LUMP-consistency test reports this class of failure.</t>
+          <t>Selected SelfTest has one active matching catalog row; selected WukongCallHome and CapabilityTest have zero. All three selected binary hashes match their files. Genesis confirms the approved Namespace list is authoritative; missing active catalog rows do not invalidate these selections. Hash agreement alone is not full execution qualification.</t>
         </is>
       </c>
       <c r="E3" s="28" t="inlineStr">
         <is>
-          <t>Review exact selected artifact versus intended revision and manifest history; propose an explicit approved reconciliation. Do not silently select latest, rewrite history or regenerate images.</t>
+          <t>Correct the test's requirement for an active manifest row and inspect consumers for equivalent catalog vetoes. Validate exact Namespace-selected bytes, identity, permissions, allocation and binding directly. A library/history index may locate files but cannot override approval. No catalog repair or reselection is required merely to satisfy this test.</t>
         </is>
       </c>
       <c r="F3" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Update lump admission service and test documentation
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
+++ b/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
@@ -6308,7 +6308,7 @@
       <c r="H70" s="28" t="inlineStr"/>
       <c r="I70" s="28" t="inlineStr">
         <is>
-          <t>Workflow snapshot reports ns-slot-modal-persist failures; no new diagnosis.</t>
+          <t>Fresh partial evidence: ADD-modal 36/36; boot-authority and single-save JavaScript checks pass. Admission no longer depends on active catalog rows. Server fixture failures and integrated browser acceptance remain; not closed.</t>
         </is>
       </c>
       <c r="J70" s="28" t="inlineStr">
@@ -6328,7 +6328,7 @@
       </c>
       <c r="M70" s="28" t="inlineStr">
         <is>
-          <t>BASE-02: docs/reviews/phase1-baseline/README.md</t>
+          <t>BASE-02: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md</t>
         </is>
       </c>
       <c r="N70" s="28" t="n"/>
@@ -6372,7 +6372,7 @@
       <c r="H71" s="28" t="inlineStr"/>
       <c r="I71" s="28" t="inlineStr">
         <is>
-          <t>Existing surfaces need integrated evidence, not generic failure alerts or inferred freshness.</t>
+          <t>Selected-file errors now distinguish unreadable and changed bytes and provide a corrective action. Integrated UI and executed-artifact freshness still need verification.</t>
         </is>
       </c>
       <c r="J71" s="28" t="inlineStr">
@@ -6390,7 +6390,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="M71" s="28" t="n"/>
+      <c r="M71" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/namespace-authority-progress.md</t>
+        </is>
+      </c>
       <c r="N71" s="28" t="n"/>
     </row>
     <row r="72" ht="90" customHeight="1" s="14">
@@ -7044,7 +7048,7 @@
       <c r="H82" s="28" t="inlineStr"/>
       <c r="I82" s="28" t="inlineStr">
         <is>
-          <t>Portable artifacts, localized C-lists and Namespace descriptors have different integrity boundaries.</t>
+          <t>Exact-byte checks retained independently of catalog status; pending bytes, changed files and immutable local derivatives tested. Full seal/replay/field coverage not established.</t>
         </is>
       </c>
       <c r="J82" s="28" t="inlineStr">
@@ -7064,7 +7068,7 @@
       </c>
       <c r="M82" s="28" t="inlineStr">
         <is>
-          <t>BASE-03: docs/reviews/phase1-baseline/README.md</t>
+          <t>BASE-03: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md</t>
         </is>
       </c>
       <c r="N82" s="28" t="n"/>
@@ -7740,7 +7744,7 @@
       <c r="H93" s="28" t="inlineStr"/>
       <c r="I93" s="28" t="inlineStr">
         <is>
-          <t>Snapshot reports LUMP consistency, boot image, endpoints, ROM guards and E2E failures; causes unverified.</t>
+          <t>Fresh R26 selected-bytes check passes; ADD-modal 36/36. Admission suite: 17 passed, 1 copied boot-fixture allocation failure. Broader diagnostic run had 91 passed/46 failed including isolation/setup failures; not release qualification.</t>
         </is>
       </c>
       <c r="J93" s="28" t="inlineStr">
@@ -7760,7 +7764,7 @@
       </c>
       <c r="M93" s="28" t="inlineStr">
         <is>
-          <t>BASE-01: docs/reviews/phase1-baseline/README.md; BASE-03: docs/reviews/phase1-baseline/README.md; BASE-08: docs/reviews/phase1-baseline/README.md</t>
+          <t>BASE-01: docs/reviews/phase1-baseline/README.md; BASE-03: docs/reviews/phase1-baseline/README.md; BASE-08: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md</t>
         </is>
       </c>
       <c r="N93" s="28" t="n"/>
@@ -8601,7 +8605,7 @@
       </c>
       <c r="F107" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G107" s="28" t="inlineStr">
@@ -8616,7 +8620,7 @@
       </c>
       <c r="I107" s="28" t="inlineStr">
         <is>
-          <t>Test imposes a competing manifest-authority requirement. Selected SelfTest has one active matching catalog row; selected WukongCallHome and CapabilityTest have zero. All three selected binary hashes match their files. Genesis confirms the approved Namespace list is authoritative; missing active catalog rows do not invalidate these selections. Hash agreement alone is not full execution qualification.</t>
+          <t>Runtime admission and R26 now validate exact Namespace-selected bytes without an active manifest-row requirement. Real admission passes with missing, archived and duplicate catalog entries. Further consumer/flow evidence remains.</t>
         </is>
       </c>
       <c r="J107" s="28" t="inlineStr">
@@ -8636,7 +8640,7 @@
       </c>
       <c r="M107" s="28" t="inlineStr">
         <is>
-          <t>docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md</t>
         </is>
       </c>
       <c r="N107" s="28" t="n"/>
@@ -9815,7 +9819,7 @@
       </c>
     </row>
     <row r="15" ht="80" customHeight="1" s="14">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Namespace authority</t>
         </is>
@@ -9932,12 +9936,12 @@
       </c>
       <c r="D3" s="28" t="inlineStr">
         <is>
-          <t>Selected SelfTest has one active matching catalog row; selected WukongCallHome and CapabilityTest have zero. All three selected binary hashes match their files. Genesis confirms the approved Namespace list is authoritative; missing active catalog rows do not invalidate these selections. Hash agreement alone is not full execution qualification.</t>
+          <t>Selected SelfTest has one active matching catalog row; selected WukongCallHome and CapabilityTest have zero. All three selected binary hashes match their files. Genesis confirms the approved Namespace list is authoritative; missing active catalog rows do not invalidate these selections. Hash agreement alone is not full execution qualification. Subsequent implementation: admission and R26 catalog veto removed; see docs/reviews/phase1-baseline/namespace-authority-progress.md</t>
         </is>
       </c>
       <c r="E3" s="28" t="inlineStr">
         <is>
-          <t>Correct the test's requirement for an active manifest row and inspect consumers for equivalent catalog vetoes. Validate exact Namespace-selected bytes, identity, permissions, allocation and binding directly. A library/history index may locate files but cannot override approval. No catalog repair or reselection is required merely to satisfy this test.</t>
+          <t>Verify remaining save/preview/image consumers against Namespace authority. Preserve exact-byte and allocation checks; no catalog repair or reselection merely for archive flags.</t>
         </is>
       </c>
       <c r="F3" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Complete isolated Namespace acceptance and exact boot revision selection
Replit-Task-Id: 666d08ab-dbd4-4316-8b66-1ba36f9a9563
Replit-Merge-Attempt: MergeTask:666d08ab-dbd4-4316-8b66-1ba36f9a9563:1:394fa12e
</commit_message>
<xml_diff>
--- a/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
+++ b/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
@@ -6297,7 +6297,7 @@
       </c>
       <c r="F70" s="28" t="inlineStr">
         <is>
-          <t>Needs verification</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G70" s="28" t="inlineStr">
@@ -6308,7 +6308,7 @@
       <c r="H70" s="28" t="inlineStr"/>
       <c r="I70" s="28" t="inlineStr">
         <is>
-          <t>Fresh partial evidence: ADD-modal 36/36; boot-authority and single-save JavaScript checks pass. Admission no longer depends on active catalog rows. Server fixture failures and integrated browser acceptance remain; not closed.</t>
+          <t>Verified: 35 extracted-route tests; 4 real isolated endpoint acceptance tests; browser cancellation/resident save-reload/stale-tab checks, then targeted passing boot and incomplete-design follow-up after exact-revision UI repair. Complete saved rows/layout/identity and protected hashes checked; all 1,280 live files byte-identical. No runtime integrity checks weakened.</t>
         </is>
       </c>
       <c r="J70" s="28" t="inlineStr">
@@ -6328,7 +6328,7 @@
       </c>
       <c r="M70" s="28" t="inlineStr">
         <is>
-          <t>BASE-02: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md</t>
+          <t>docs/reviews/phase1-baseline/namespace-authority-progress.md#final-closure-evidence; scripts/run_namespace_save_acceptance.py; tests/e2e/namespace_save_acceptance.spec.js</t>
         </is>
       </c>
       <c r="N70" s="28" t="n"/>

</xml_diff>

<commit_message>
Update agent metadata and automate phase 1 progress tracking
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
+++ b/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
@@ -7424,7 +7424,7 @@
       <c r="H88" s="28" t="inlineStr"/>
       <c r="I88" s="28" t="inlineStr">
         <is>
-          <t>Current fixtures and legacy saved image layouts differ; no silent binary reinterpretation.</t>
+          <t>Fresh combined verification: resident addresses 1024/7872, complete body identity, Thread ranges, matching Step-2 placements and private simulation checks pass without xfail exemptions. This is image-generator evidence only; same-byte simulator/RTL instruction conformance remains unverified.</t>
         </is>
       </c>
       <c r="J88" s="28" t="inlineStr">
@@ -7444,7 +7444,7 @@
       </c>
       <c r="M88" s="28" t="inlineStr">
         <is>
-          <t>BASE-04: docs/reviews/phase1-baseline/README.md; BASE-05: docs/reviews/phase1-baseline/README.md</t>
+          <t>BASE-04: docs/reviews/phase1-baseline/README.md; BASE-05: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md#combined-post-merge-verification--17-october-2026</t>
         </is>
       </c>
       <c r="N88" s="28" t="n"/>
@@ -7744,7 +7744,7 @@
       <c r="H93" s="28" t="inlineStr"/>
       <c r="I93" s="28" t="inlineStr">
         <is>
-          <t>Fresh R26 selected-bytes check passes; ADD-modal 36/36. Admission suite: 17 passed, 1 copied boot-fixture allocation failure. Broader diagnostic run had 91 passed/46 failed including isolation/setup failures; not release qualification.</t>
+          <t>Fresh combined merge verification: 190 passed, 2 failed; no skips/xfails. Admission/allocation/private simulation: 128 passes. Independent image suite: 62 passes, 2 migration failures (parent/explicit config). Historical migration copies device address 0x40000014 into resident NS[10]; generator correctly rejects out-of-RAM placement. Other regression groups remain open.</t>
         </is>
       </c>
       <c r="J93" s="28" t="inlineStr">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="M93" s="28" t="inlineStr">
         <is>
-          <t>BASE-01: docs/reviews/phase1-baseline/README.md; BASE-03: docs/reviews/phase1-baseline/README.md; BASE-08: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md</t>
+          <t>BASE-01: docs/reviews/phase1-baseline/README.md; BASE-03: docs/reviews/phase1-baseline/README.md; BASE-08: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md; docs/reviews/phase1-baseline/namespace-authority-progress.md#combined-post-merge-verification--17-october-2026</t>
         </is>
       </c>
       <c r="N93" s="28" t="n"/>
@@ -9204,7 +9204,7 @@
       </c>
       <c r="B3" s="28">
         <f>COUNTA(Completeness!A2:A10000)</f>
-        <v/>
+        <v>113</v>
       </c>
       <c r="C3" s="28" t="n"/>
       <c r="D3" s="28" t="n"/>
@@ -9217,7 +9217,7 @@
       </c>
       <c r="B4" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Open")</f>
-        <v/>
+        <v>24</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="B5" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="C5" s="28" t="n"/>
       <c r="D5" s="28" t="n"/>
@@ -9243,7 +9243,7 @@
       </c>
       <c r="B6" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Not run")</f>
-        <v/>
+        <v>56</v>
       </c>
       <c r="C6" s="28" t="n"/>
       <c r="D6" s="28" t="n"/>
@@ -9256,7 +9256,7 @@
       </c>
       <c r="B7" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Needs verification")</f>
-        <v/>
+        <v>24</v>
       </c>
       <c r="C7" s="28" t="n"/>
       <c r="D7" s="28" t="n"/>
@@ -9269,7 +9269,7 @@
       </c>
       <c r="B8" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"In progress")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C8" s="28" t="n"/>
       <c r="D8" s="28" t="n"/>
@@ -9282,7 +9282,7 @@
       </c>
       <c r="B9" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="C9" s="28" t="n"/>
       <c r="D9" s="28" t="n"/>
@@ -9295,7 +9295,7 @@
       </c>
       <c r="B10" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Failed")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C10" s="28" t="n"/>
       <c r="D10" s="28" t="n"/>
@@ -9308,7 +9308,7 @@
       </c>
       <c r="B11" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Out of scope")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="C11" s="28" t="n"/>
       <c r="D11" s="28" t="n"/>
@@ -9321,7 +9321,7 @@
       </c>
       <c r="B12" s="29">
         <f>IFERROR(COUNTIF(Completeness!F2:F10000,"Complete")/(COUNTA(Completeness!A2:A10000)-COUNTIF(Completeness!F2:F10000,"Out of scope")),0)</f>
-        <v/>
+        <v>0.017857142857142856</v>
       </c>
       <c r="C12" s="28" t="n"/>
       <c r="D12" s="28" t="n"/>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="B13" s="28" t="inlineStr">
         <is>
-          <t>Unweighted row closure, NOT percentage of ISA/security proved. Software gaps are not automatically bitstream gates.</t>
+          <t>Counts of different items; each item has one status. Row completion is not ISA/security coverage.</t>
         </is>
       </c>
       <c r="C13" s="28" t="n"/>
@@ -9353,12 +9353,12 @@
       </c>
       <c r="C14" s="28" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Complete items</t>
         </is>
       </c>
       <c r="D14" s="28" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Blocked items</t>
         </is>
       </c>
     </row>
@@ -9370,15 +9370,15 @@
       </c>
       <c r="B15" s="28">
         <f>COUNTIF(Completeness!B2:B10000,A15)</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="C15" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A15,Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D15" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A15,Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1" s="14">
@@ -9389,15 +9389,15 @@
       </c>
       <c r="B16" s="28">
         <f>COUNTIF(Completeness!B2:B10000,A16)</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="C16" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A16,Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D16" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A16,Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1" s="14">
@@ -9408,15 +9408,15 @@
       </c>
       <c r="B17" s="28">
         <f>COUNTIF(Completeness!B2:B10000,A17)</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="C17" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A17,Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="D17" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A17,Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="18" ht="48" customHeight="1" s="14">
@@ -9427,15 +9427,15 @@
       </c>
       <c r="B18" s="28">
         <f>COUNTIF(Completeness!B2:B10000,A18)</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="C18" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A18,Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D18" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A18,Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="19" ht="48" customHeight="1" s="14">
@@ -9446,15 +9446,15 @@
       </c>
       <c r="B19" s="28">
         <f>COUNTIF(Completeness!B2:B10000,A19)</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="C19" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A19,Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D19" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A19,Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="20" ht="48" customHeight="1" s="14">
@@ -9465,15 +9465,15 @@
       </c>
       <c r="B20" s="28">
         <f>COUNTIF(Completeness!B2:B10000,A20)</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="C20" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A20,Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D20" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A20,Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="21" ht="48" customHeight="1" s="14">
@@ -9484,15 +9484,15 @@
       </c>
       <c r="B21" s="28">
         <f>COUNTIF(Completeness!B2:B10000,A21)</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="C21" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A21,Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D21" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A21,Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="22" ht="48" customHeight="1" s="14">
@@ -9503,15 +9503,15 @@
       </c>
       <c r="B22" s="28">
         <f>COUNTIF(Completeness!B2:B10000,A22)</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="C22" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A22,Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D22" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A22,Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="23" ht="48" customHeight="1" s="14">
@@ -9522,15 +9522,15 @@
       </c>
       <c r="B23" s="28">
         <f>COUNTIF(Completeness!B2:B10000,A23)</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="C23" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A23,Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D23" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A23,Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="24" ht="48" customHeight="1" s="14">
@@ -9541,15 +9541,15 @@
       </c>
       <c r="B24" s="28">
         <f>COUNTIF(Completeness!B2:B10000,A24)</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="C24" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A24,Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D24" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A24,Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="25" ht="48" customHeight="1" s="14">
@@ -9560,15 +9560,15 @@
       </c>
       <c r="B25" s="28">
         <f>COUNTIF(Completeness!B2:B10000,A25)</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="C25" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A25,Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D25" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A25,Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="26" ht="48" customHeight="1" s="14">
@@ -9579,15 +9579,15 @@
       </c>
       <c r="B26" s="28">
         <f>COUNTIF(Completeness!B2:B10000,A26)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="C26" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A26,Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="D26" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A26,Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="27" ht="48" customHeight="1" s="14">
@@ -9598,15 +9598,15 @@
       </c>
       <c r="B27" s="28">
         <f>COUNTIF(Completeness!B2:B10000,A27)</f>
-        <v/>
+        <v>15</v>
       </c>
       <c r="C27" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A27,Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D27" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A27,Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -9617,15 +9617,15 @@
       </c>
       <c r="B28" s="28">
         <f>COUNTIF(Completeness!B2:B10000,A28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="C28" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A28,Completeness!F2:F10000,"Complete")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D28" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A28,Completeness!F2:F10000,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update agent configuration and document phase one review progress
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
+++ b/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Progress" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Tracking guide" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Baseline audit" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Approved target" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Threat Map'!$A$5:$M$20</definedName>
@@ -24,6 +25,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tracking guide'!$A$1:$B$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Tracking guide'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Baseline audit'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Approved target'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -161,7 +163,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -246,6 +248,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,6 +427,18 @@
     <tableColumn id="4" name="Observation"/>
     <tableColumn id="5" name="Next action"/>
     <tableColumn id="6" name="Related requirements"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Phase1ApprovedTarget" displayName="Phase1ApprovedTarget" ref="A1:C19" headerRowCount="1">
+  <autoFilter ref="A1:C19"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Slot"/>
+    <tableColumn id="2" name="Approved entry"/>
+    <tableColumn id="3" name="Design intent"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -6297,7 +6314,7 @@
       </c>
       <c r="F70" s="28" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G70" s="28" t="inlineStr">
@@ -6308,7 +6325,7 @@
       <c r="H70" s="28" t="inlineStr"/>
       <c r="I70" s="28" t="inlineStr">
         <is>
-          <t>Verified: 35 extracted-route tests; 4 real isolated endpoint acceptance tests; browser cancellation/resident save-reload/stale-tab checks, then targeted passing boot and incomplete-design follow-up after exact-revision UI repair. Complete saved rows/layout/identity and protected hashes checked; all 1,280 live files byte-identical. No runtime integrity checks weakened.</t>
+          <t>Historical saved-Namespace acceptance passed, but did not exercise the Genesis-confirmed Phase 1 256-slot design (metadata 0, self 1, entry Thread 2, UART 8, CapabilityTest boot 10; all Resident). Retain old-profile evidence; verify the approved target before closure.</t>
         </is>
       </c>
       <c r="J70" s="28" t="inlineStr">
@@ -6328,7 +6345,7 @@
       </c>
       <c r="M70" s="28" t="inlineStr">
         <is>
-          <t>docs/reviews/phase1-baseline/namespace-authority-progress.md#final-closure-evidence; scripts/run_namespace_save_acceptance.py; tests/e2e/namespace_save_acceptance.spec.js</t>
+          <t>docs/reviews/phase1-baseline/namespace-authority-progress.md#final-closure-evidence; scripts/run_namespace_save_acceptance.py; tests/e2e/namespace_save_acceptance.spec.js; docs/reviews/phase1-baseline/approved-target-namespace.md</t>
         </is>
       </c>
       <c r="N70" s="28" t="n"/>
@@ -9256,7 +9273,7 @@
       </c>
       <c r="B7" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Needs verification")</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C7" s="28" t="n"/>
       <c r="D7" s="28" t="n"/>
@@ -9282,7 +9299,7 @@
       </c>
       <c r="B9" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Complete")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="28" t="n"/>
       <c r="D9" s="28" t="n"/>
@@ -9321,7 +9338,7 @@
       </c>
       <c r="B12" s="29">
         <f>IFERROR(COUNTIF(Completeness!F2:F10000,"Complete")/(COUNTA(Completeness!A2:A10000)-COUNTIF(Completeness!F2:F10000,"Out of scope")),0)</f>
-        <v>0.017857142857142856</v>
+        <v>0.008928571428571428</v>
       </c>
       <c r="C12" s="28" t="n"/>
       <c r="D12" s="28" t="n"/>
@@ -9412,7 +9429,7 @@
       </c>
       <c r="C17" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A17,Completeness!F2:F10000,"Complete")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D17" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A17,Completeness!F2:F10000,"Blocked")</f>
@@ -9641,7 +9658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" style="14" min="1" max="1"/>
@@ -9827,6 +9844,18 @@
       <c r="B15" s="28" t="inlineStr">
         <is>
           <t>Genesis-approved Namespace selection is authoritative. A manifest may index library/history files, but missing, archived or duplicate catalog rows cannot veto independently verified selected bytes. BASE-02 tracks the competing test requirement, not a request to repair approved selections.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Approved Phase 1 target</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Use Approved target and docs/reviews/phase1-baseline/approved-target-namespace.md. IDE-03 legacy-profile evidence is not acceptance of this target. Code work is linked through original requirement IDs; merged coding tasks do not automatically close those requirements.</t>
         </is>
       </c>
     </row>
@@ -10181,4 +10210,419 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:C27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" style="14" min="1" max="1"/>
+    <col width="30" customWidth="1" style="14" min="2" max="2"/>
+    <col width="65" customWidth="1" style="14" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="B1" s="30" t="inlineStr">
+        <is>
+          <t>Approved entry</t>
+        </is>
+      </c>
+      <c r="C1" s="30" t="inlineStr">
+        <is>
+          <t>Design intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" s="28" t="inlineStr">
+        <is>
+          <t>Namespace metadata/header</t>
+        </is>
+      </c>
+      <c r="C2" s="28" t="inlineStr">
+        <is>
+          <t>Four-word table metadata</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>Boot.NS</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>Namespace self; Resident</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Boot.Thread</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>Entry Thread; Resident</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>LED_DEV</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>Resident I/O register</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>BTN_DEV</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>Resident I/O register</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>TIMER_DEV</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr">
+        <is>
+          <t>Resident I/O register</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>SelfTest</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>Resident</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="28" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>WukongCallHome</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="inlineStr">
+        <is>
+          <t>Resident</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>UART_DEV</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="inlineStr">
+        <is>
+          <t>Resident I/O register</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="28" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>ide.Mint</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="inlineStr">
+        <is>
+          <t>Resident intent; unfinished implementation retained</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="28" t="inlineStr">
+        <is>
+          <t>CapabilityTest</t>
+        </is>
+      </c>
+      <c r="C12" s="28" t="inlineStr">
+        <is>
+          <t>Resident; selected boot entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="28" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>Thread.2</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="inlineStr">
+        <is>
+          <t>Resident Thread</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="28" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>Thread.3</t>
+        </is>
+      </c>
+      <c r="C14" s="28" t="inlineStr">
+        <is>
+          <t>Resident Thread</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="28" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>M_BIT_DEV</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>Resident I/O register</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="28" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>nstab</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>Resident intent; requested RW</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="28" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>pkverify</t>
+        </is>
+      </c>
+      <c r="C17" s="28" t="inlineStr">
+        <is>
+          <t>Resident intent; requested E</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="28" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>ide.Alice</t>
+        </is>
+      </c>
+      <c r="C18" s="28" t="inlineStr">
+        <is>
+          <t>Resident intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="28" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>ide.Mallory</t>
+        </is>
+      </c>
+      <c r="C19" s="28" t="inlineStr">
+        <is>
+          <t>Resident intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="n"/>
+      <c r="B20" s="28" t="n"/>
+      <c r="C20" s="28" t="n"/>
+    </row>
+    <row r="21" ht="44" customHeight="1" s="14">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="B21" s="28" t="inlineStr">
+        <is>
+          <t>2026-10-17; Genesis explicitly approved the pictured Phase 1 design.</t>
+        </is>
+      </c>
+      <c r="C21" s="28" t="n"/>
+    </row>
+    <row r="22" ht="44" customHeight="1" s="14">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="B22" s="28" t="inlineStr">
+        <is>
+          <t>256 total slots including metadata; 1024 words / 4096 bytes; table-only CR15 limit 1023.</t>
+        </is>
+      </c>
+      <c r="C22" s="28" t="n"/>
+    </row>
+    <row r="23" ht="44" customHeight="1" s="14">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>Policy</t>
+        </is>
+      </c>
+      <c r="B23" s="28" t="inlineStr">
+        <is>
+          <t>17 assigned entries, all Resident intent; no Lazy placements. IDE node: ide.</t>
+        </is>
+      </c>
+      <c r="C23" s="28" t="n"/>
+    </row>
+    <row r="24" ht="44" customHeight="1" s="14">
+      <c r="A24" s="28" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B24" s="28" t="inlineStr">
+        <is>
+          <t>Design confirmation only; no installation, activation, live migration or hardware actions.</t>
+        </is>
+      </c>
+      <c r="C24" s="28" t="n"/>
+    </row>
+    <row r="25" ht="44" customHeight="1" s="14">
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>Acceptance</t>
+        </is>
+      </c>
+      <c r="B25" s="28" t="inlineStr">
+        <is>
+          <t>IDE-03 is Needs verification against this target. Older-profile passing results remain historical evidence.</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="n"/>
+    </row>
+    <row r="26" ht="44" customHeight="1" s="14">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>Coding work</t>
+        </is>
+      </c>
+      <c r="B26" s="28" t="inlineStr">
+        <is>
+          <t>Completeness includes implementation requirements, not a one-to-one project-task queue. Each code task should reference its requirement IDs and this target.</t>
+        </is>
+      </c>
+      <c r="C26" s="28" t="n"/>
+    </row>
+    <row r="27" ht="44" customHeight="1" s="14">
+      <c r="A27" s="28" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="B27" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/phase1-baseline/approved-target-namespace.md</t>
+        </is>
+      </c>
+      <c r="C27" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Verify approved Phase 1 Namespace save/reload and close original IDE-03
Replit-Task-Id: 416bba13-aa85-4e28-940f-091c4f4ed818
Replit-Merge-Attempt: MergeTask:416bba13-aa85-4e28-940f-091c4f4ed818:1:47905561
</commit_message>
<xml_diff>
--- a/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
+++ b/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
@@ -6314,7 +6314,7 @@
       </c>
       <c r="F70" s="28" t="inlineStr">
         <is>
-          <t>Needs verification</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G70" s="28" t="inlineStr">
@@ -6325,7 +6325,7 @@
       <c r="H70" s="28" t="inlineStr"/>
       <c r="I70" s="28" t="inlineStr">
         <is>
-          <t>Historical saved-Namespace acceptance passed, but did not exercise the Genesis-confirmed Phase 1 256-slot design (metadata 0, self 1, entry Thread 2, UART 8, CapabilityTest boot 10; all Resident). Retain old-profile evidence; verify the approved target before closure.</t>
+          <t>Approved Phase 1 256-slot profile accepted through original controls and actual isolated endpoints: exact revisions, 17 Resident-intent entries/no Lazy, unfinished rows, edits/save/reload, cancellation, boot 7→10 and cross-profile isolation. 4 endpoint + 26 focused server checks passed. Browser journey completed in targeted segments after two test-only assumptions were corrected; no fresh full-command green run claimed. 1,281 live artifact/configuration files unchanged. Historical results retained; no execution/hardware qualification.</t>
         </is>
       </c>
       <c r="J70" s="28" t="inlineStr">
@@ -6345,7 +6345,7 @@
       </c>
       <c r="M70" s="28" t="inlineStr">
         <is>
-          <t>docs/reviews/phase1-baseline/namespace-authority-progress.md#final-closure-evidence; scripts/run_namespace_save_acceptance.py; tests/e2e/namespace_save_acceptance.spec.js; docs/reviews/phase1-baseline/approved-target-namespace.md</t>
+          <t>docs/reviews/phase1-baseline/namespace-authority-progress.md#final-closure-evidence; scripts/run_namespace_save_acceptance.py; tests/e2e/namespace_save_acceptance.spec.js; docs/reviews/phase1-baseline/approved-target-namespace.md; docs/reviews/phase1-baseline/phase1-save-reload-acceptance.md; tests/fixtures/phase1_namespace_target.json; tests/e2e/namespace_phase1_acceptance.spec.js</t>
         </is>
       </c>
       <c r="N70" s="28" t="n"/>
@@ -9273,7 +9273,7 @@
       </c>
       <c r="B7" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Needs verification")</f>
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C7" s="28" t="n"/>
       <c r="D7" s="28" t="n"/>
@@ -9299,7 +9299,7 @@
       </c>
       <c r="B9" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Complete")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" s="28" t="n"/>
       <c r="D9" s="28" t="n"/>
@@ -9338,7 +9338,7 @@
       </c>
       <c r="B12" s="29">
         <f>IFERROR(COUNTIF(Completeness!F2:F10000,"Complete")/(COUNTA(Completeness!A2:A10000)-COUNTIF(Completeness!F2:F10000,"Out of scope")),0)</f>
-        <v>0.008928571428571428</v>
+        <v>0.017857142857142856</v>
       </c>
       <c r="C12" s="28" t="n"/>
       <c r="D12" s="28" t="n"/>
@@ -9429,7 +9429,7 @@
       </c>
       <c r="C17" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A17,Completeness!F2:F10000,"Complete")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A17,Completeness!F2:F10000,"Blocked")</f>
@@ -9848,12 +9848,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>Approved Phase 1 target</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Use Approved target and docs/reviews/phase1-baseline/approved-target-namespace.md. IDE-03 legacy-profile evidence is not acceptance of this target. Code work is linked through original requirement IDs; merged coding tasks do not automatically close those requirements.</t>
         </is>
@@ -10529,7 +10529,6 @@
           <t>2026-10-17; Genesis explicitly approved the pictured Phase 1 design.</t>
         </is>
       </c>
-      <c r="C21" s="28" t="n"/>
     </row>
     <row r="22" ht="44" customHeight="1" s="14">
       <c r="A22" s="28" t="inlineStr">
@@ -10542,7 +10541,6 @@
           <t>256 total slots including metadata; 1024 words / 4096 bytes; table-only CR15 limit 1023.</t>
         </is>
       </c>
-      <c r="C22" s="28" t="n"/>
     </row>
     <row r="23" ht="44" customHeight="1" s="14">
       <c r="A23" s="28" t="inlineStr">
@@ -10555,7 +10553,6 @@
           <t>17 assigned entries, all Resident intent; no Lazy placements. IDE node: ide.</t>
         </is>
       </c>
-      <c r="C23" s="28" t="n"/>
     </row>
     <row r="24" ht="44" customHeight="1" s="14">
       <c r="A24" s="28" t="inlineStr">
@@ -10568,7 +10565,6 @@
           <t>Design confirmation only; no installation, activation, live migration or hardware actions.</t>
         </is>
       </c>
-      <c r="C24" s="28" t="n"/>
     </row>
     <row r="25" ht="44" customHeight="1" s="14">
       <c r="A25" s="28" t="inlineStr">
@@ -10581,7 +10577,6 @@
           <t>IDE-03 is Needs verification against this target. Older-profile passing results remain historical evidence.</t>
         </is>
       </c>
-      <c r="C25" s="28" t="n"/>
     </row>
     <row r="26" ht="44" customHeight="1" s="14">
       <c r="A26" s="28" t="inlineStr">
@@ -10594,7 +10589,6 @@
           <t>Completeness includes implementation requirements, not a one-to-one project-task queue. Each code task should reference its requirement IDs and this target.</t>
         </is>
       </c>
-      <c r="C26" s="28" t="n"/>
     </row>
     <row r="27" ht="44" customHeight="1" s="14">
       <c r="A27" s="28" t="inlineStr">
@@ -10607,7 +10601,6 @@
           <t>docs/reviews/phase1-baseline/approved-target-namespace.md</t>
         </is>
       </c>
-      <c r="C27" s="28" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
Update agent metadata, test plan, and W7 review script
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
+++ b/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
@@ -1906,7 +1906,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="F2" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G2" s="28" t="inlineStr">
@@ -2041,12 +2041,14 @@
       <c r="H2" s="28" t="inlineStr"/>
       <c r="I2" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Recorded full-core RTL CREATE/DESTROY cases reject captured old GTs after release and reuse; slot tests cover version boundaries. Partial RTL-model evidence, not physical-board timing.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J2" s="28" t="inlineStr">
         <is>
-          <t>Make N copies of a GT; revoke once. Every copy faults; revoke cost independent of N (FPGA cycle counter). Coverage: Sweep N = 1…max c-list size; cycle count must be flat</t>
+          <t>Make N copies of a GT; revoke once. Every copy faults; revoke cost independent of N (FPGA cycle counter). Coverage: Sweep N = 1…max c-list size; cycle count must be flat
+Review action: Run copied-GT N sweep, generation-boundary coverage and FPGA cycle-cost measurements; identify exact authorized revoke operation.</t>
         </is>
       </c>
       <c r="K2" s="28" t="inlineStr">
@@ -2056,10 +2058,14 @@
       </c>
       <c r="L2" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M2" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M2" s="28" t="inlineStr">
+        <is>
+          <t>docs/phase-1/mint-destroy-v1-development.md; docs/phase-1/mint-slot-package.md</t>
+        </is>
+      </c>
       <c r="N2" s="28" t="n"/>
     </row>
     <row r="3" ht="90" customHeight="1" s="14">
@@ -2090,7 +2096,7 @@
       </c>
       <c r="F3" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G3" s="28" t="inlineStr">
@@ -2101,12 +2107,14 @@
       <c r="H3" s="28" t="inlineStr"/>
       <c r="I3" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): 2026-10-20 saved Alice/Mallory image: Alice stores/retrieves 731; Mallory first faults NO_CAPABILITY at LOAD PC 1 before DREAD; Alice body unchanged. Mint adds focused identity/version checks.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J3" s="28" t="inlineStr">
         <is>
-          <t>Forged bit patterns, data-as-capability, out-of-bounds offsets all fault. Coverage: Exhaustive over typ / tag / version fields; structured fuzz over offsets</t>
+          <t>Forged bit patterns, data-as-capability, out-of-bounds offsets all fault. Coverage: Exhaustive over typ / tag / version fields; structured fuzz over offsets
+Review action: Complete exhaustive typ/tag/version and structured offset coverage, plus exact-board evidence. Missing-row denial alone is not forged-reference closure.</t>
         </is>
       </c>
       <c r="K3" s="28" t="inlineStr">
@@ -2116,10 +2124,14 @@
       </c>
       <c r="L3" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M3" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M3" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/saved-alice-mallory-execution.md; docs/phase-1/mint-destroy-v1-development.md</t>
+        </is>
+      </c>
       <c r="N3" s="28" t="n"/>
     </row>
     <row r="4" ht="90" customHeight="1" s="14">
@@ -2161,12 +2173,14 @@
       <c r="H4" s="28" t="inlineStr"/>
       <c r="I4" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): No completed actual-production-root closure proof identified in reviewed evidence.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J4" s="28" t="inlineStr">
         <is>
-          <t>Reachability closure from prod root contains no debug authority. Coverage: Graph closure over all c-lists reachable from prod root</t>
+          <t>Reachability closure from prod root contains no debug authority. Coverage: Graph closure over all c-lists reachable from prod root
+Review action: Analyze production root, dynamic grants and loading assumptions; retain W7 baseline requirement for comparative claims.</t>
         </is>
       </c>
       <c r="K4" s="28" t="inlineStr">
@@ -2176,10 +2190,14 @@
       </c>
       <c r="L4" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M4" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M4" s="28" t="inlineStr">
+        <is>
+          <t>docs/phase-1/W7-plus-plus-test-objectives.md</t>
+        </is>
+      </c>
       <c r="N4" s="28" t="n"/>
     </row>
     <row r="5" ht="90" customHeight="1" s="14">
@@ -2210,7 +2228,7 @@
       </c>
       <c r="F5" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G5" s="28" t="inlineStr">
@@ -2221,12 +2239,14 @@
       <c r="H5" s="28" t="inlineStr"/>
       <c r="I5" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Native Mint and full-core RTL lifecycle reports provide allocation/issued-GT evidence. Private provisioning and permissive PkVerify are explicit test restrictions.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J5" s="28" t="inlineStr">
         <is>
-          <t>Newborn lump's reachable authority equals exactly what the womb granted. Coverage: Authority census at birth for every lump type</t>
+          <t>Newborn lump's reachable authority equals exactly what the womb granted. Coverage: Authority census at birth for every lump type
+Review action: Complete birth-authority census for each type and operational requester/proof enforcement; do not credit test authorization as production security.</t>
         </is>
       </c>
       <c r="K5" s="28" t="inlineStr">
@@ -2236,10 +2256,14 @@
       </c>
       <c r="L5" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M5" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M5" s="28" t="inlineStr">
+        <is>
+          <t>docs/phase-1/mint-destroy-v1-development.md; docs/reviews/mint-phase1/native-lambda-binding.md</t>
+        </is>
+      </c>
       <c r="N5" s="28" t="n"/>
     </row>
     <row r="6" ht="90" customHeight="1" s="14">
@@ -2270,7 +2294,7 @@
       </c>
       <c r="F6" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G6" s="28" t="inlineStr">
@@ -2281,12 +2305,14 @@
       <c r="H6" s="28" t="inlineStr"/>
       <c r="I6" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Exact-byte compiler/save and destination checks provide supporting integrity evidence, not unsealer or cross-Namespace acceptance.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J6" s="28" t="inlineStr">
         <is>
-          <t>Unseal without unsealer faults; exporting an Abstract GT across namespaces faults. Coverage: Exhaustive over namespace pairs</t>
+          <t>Unseal without unsealer faults; exporting an Abstract GT across namespaces faults. Coverage: Exhaustive over namespace pairs
+Review action: Reconcile sealing/type oracle; test unauthorized unseal and qualified Namespace pairs. Keep Phase 2 dependencies explicit.</t>
         </is>
       </c>
       <c r="K6" s="28" t="inlineStr">
@@ -2296,10 +2322,14 @@
       </c>
       <c r="L6" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M6" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M6" s="28" t="inlineStr">
+        <is>
+          <t>tests/server/test_named_call_save_attestation.py; docs/phase-1/W7-plus-plus-test-objectives.md</t>
+        </is>
+      </c>
       <c r="N6" s="28" t="n"/>
     </row>
     <row r="7" ht="90" customHeight="1" s="14">
@@ -2330,7 +2360,7 @@
       </c>
       <c r="F7" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G7" s="28" t="inlineStr">
@@ -2341,12 +2371,14 @@
       <c r="H7" s="28" t="inlineStr"/>
       <c r="I7" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Cleaner component/lifecycle tests cover allocation, clearing, reuse and exhaustion under isolated provisioning.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J7" s="28" t="inlineStr">
         <is>
-          <t>Hostile namespace allocates unboundedly; neighbours see no failure and latency within stated bound. Coverage: Stress test across namespace counts</t>
+          <t>Hostile namespace allocates unboundedly; neighbours see no failure and latency within stated bound. Coverage: Stress test across namespace counts
+Review action: Define and measure enforceable resource/latency bounds and neighbor isolation; do not assume tracing GC or eviction.</t>
         </is>
       </c>
       <c r="K7" s="28" t="inlineStr">
@@ -2356,10 +2388,14 @@
       </c>
       <c r="L7" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M7" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M7" s="28" t="inlineStr">
+        <is>
+          <t>docs/phase-1/mint-destroy-v1-development.md; docs/phase-1/W7-plus-plus-test-objectives.md</t>
+        </is>
+      </c>
       <c r="N7" s="28" t="n"/>
     </row>
     <row r="8" ht="90" customHeight="1" s="14">
@@ -2390,7 +2426,7 @@
       </c>
       <c r="F8" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G8" s="28" t="inlineStr">
@@ -2401,12 +2437,14 @@
       <c r="H8" s="28" t="inlineStr"/>
       <c r="I8" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Saved-design execution and exact-byte Save checks demonstrate partial persistence-path behavior. Prior session: five named-CALL save tests passed in isolated repositories.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J8" s="28" t="inlineStr">
         <is>
-          <t>Evict, reload, compare authority: identical; no file-system path involved. Coverage: Round-trip every lump type</t>
+          <t>Evict, reload, compare authority: identical; no file-system path involved. Coverage: Round-trip every lump type
+Review action: Cover relevant artifact types and authority-preserving lifecycle/reset durability; file publication is not secure eviction/reload acceptance.</t>
         </is>
       </c>
       <c r="K8" s="28" t="inlineStr">
@@ -2416,10 +2454,14 @@
       </c>
       <c r="L8" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M8" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M8" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/saved-alice-mallory-execution.md; tests/server/test_named_call_save_attestation.py; docs/phase-1/mint-create-cut-points.md</t>
+        </is>
+      </c>
       <c r="N8" s="28" t="n"/>
     </row>
     <row r="9" ht="90" customHeight="1" s="14">
@@ -2461,12 +2503,14 @@
       <c r="H9" s="28" t="inlineStr"/>
       <c r="I9" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): No qualifying depth-independent elapsed-time result identified in reviewed evidence.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J9" s="28" t="inlineStr">
         <is>
-          <t>Callee loops or nests deeply; caller regains control in bounded time independent of depth. Coverage: Sweep nesting depth; response time must be flat</t>
+          <t>Callee loops or nests deeply; caller regains control in bounded time independent of depth. Coverage: Sweep nesting depth; response time must be flat
+Review action: Define fault-stop versus return-to-caller promise and measure bounded behavior across nesting depths.</t>
         </is>
       </c>
       <c r="K9" s="28" t="inlineStr">
@@ -2476,10 +2520,14 @@
       </c>
       <c r="L9" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M9" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M9" s="28" t="inlineStr">
+        <is>
+          <t>docs/phase-1/W7-plus-plus-test-objectives.md</t>
+        </is>
+      </c>
       <c r="N9" s="28" t="n"/>
     </row>
     <row r="10" ht="90" customHeight="1" s="14">
@@ -2510,7 +2558,7 @@
       </c>
       <c r="F10" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G10" s="28" t="inlineStr">
@@ -2521,12 +2569,14 @@
       <c r="H10" s="28" t="inlineStr"/>
       <c r="I10" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Native LAMBDA entry/return implementation evidence exists; LAMBDA RETURN preserves current CRs. This does not qualify retained checkpoints.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J10" s="28" t="inlineStr">
         <is>
-          <t>Callee retains its return path and invokes it twice; second call faults. Coverage: All return paths</t>
+          <t>Callee retains its return path and invokes it twice; second call faults. Coverage: All return paths
+Review action: Verify one-shot checkpoint identity, copied handles and reset lifetime separately from ordinary CALL/RETURN.</t>
         </is>
       </c>
       <c r="K10" s="28" t="inlineStr">
@@ -2536,10 +2586,14 @@
       </c>
       <c r="L10" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M10" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M10" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/mint-phase1/native-lambda-binding.md; docs/phase-1/W7-plus-plus-test-objectives.md</t>
+        </is>
+      </c>
       <c r="N10" s="28" t="n"/>
     </row>
     <row r="11" ht="90" customHeight="1" s="14">
@@ -2581,12 +2635,14 @@
       <c r="H11" s="28" t="inlineStr"/>
       <c r="I11" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Sequential private Mint lifecycle tests do not establish concurrency. Cut-point report records restored ABA and incomplete exclusion evidence.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J11" s="28" t="inlineStr">
         <is>
-          <t>Racing writers to a shared lump: serialized or faulted. Coverage: Randomised interleavings</t>
+          <t>Racing writers to a shared lump: serialized or faulted. Coverage: Randomised interleavings
+Review action: Define allowed concurrency and prove whole-update exclusion/interruption semantics. Do not count sequential lifecycle tests as concurrency acceptance.</t>
         </is>
       </c>
       <c r="K11" s="28" t="inlineStr">
@@ -2596,10 +2652,14 @@
       </c>
       <c r="L11" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M11" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M11" s="28" t="inlineStr">
+        <is>
+          <t>docs/phase-1/mint-destroy-v1-development.md; docs/phase-1/mint-create-cut-points.md</t>
+        </is>
+      </c>
       <c r="N11" s="28" t="n"/>
     </row>
     <row r="12" ht="90" customHeight="1" s="14">
@@ -2630,7 +2690,7 @@
       </c>
       <c r="F12" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G12" s="28" t="inlineStr">
@@ -2641,12 +2701,14 @@
       <c r="H12" s="28" t="inlineStr"/>
       <c r="I12" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Exact artifact/image identities and first-fault attribution are recorded for the saved actor demonstration; this is supporting evidence only.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J12" s="28" t="inlineStr">
         <is>
-          <t>Every invocation attributable to originating womb. Coverage: Trace every call chain in test suite</t>
+          <t>Every invocation attributable to originating womb. Coverage: Trace every call chain in test suite
+Review action: Define originating principal and permitted transformations; verify attribution through complete call chains.</t>
         </is>
       </c>
       <c r="K12" s="28" t="inlineStr">
@@ -2656,10 +2718,14 @@
       </c>
       <c r="L12" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M12" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M12" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/saved-alice-mallory-execution.md; docs/phase-1/W7-plus-plus-test-objectives.md</t>
+        </is>
+      </c>
       <c r="N12" s="28" t="n"/>
     </row>
     <row r="13" ht="90" customHeight="1" s="14">
@@ -2690,7 +2756,7 @@
       </c>
       <c r="F13" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G13" s="28" t="inlineStr">
@@ -2701,12 +2767,14 @@
       <c r="H13" s="28" t="inlineStr"/>
       <c r="I13" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Saved actor demonstration proves one unauthorized access attempt is stopped without changing Alice; no whole-callee leakage proof.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J13" s="28" t="inlineStr">
         <is>
-          <t>Reachability: callee holds no outward write authority at entry. Coverage: Closure over callee c-list</t>
+          <t>Reachability: callee holds no outward write authority at entry. Coverage: Closure over callee c-list
+Review action: Analyze outward authority and explicit channels over the whole callee; retain timing/covert-channel exclusions.</t>
         </is>
       </c>
       <c r="K13" s="28" t="inlineStr">
@@ -2716,10 +2784,14 @@
       </c>
       <c r="L13" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M13" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M13" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/saved-alice-mallory-execution.md; docs/phase-1/W7-plus-plus-test-objectives.md</t>
+        </is>
+      </c>
       <c r="N13" s="28" t="n"/>
     </row>
     <row r="14" ht="90" customHeight="1" s="14">
@@ -2761,12 +2833,14 @@
       <c r="H14" s="28" t="inlineStr"/>
       <c r="I14" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Limitation/trust-assumption disposition, not an executable acceptance test. Original worksheet claims and statuses retained.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J14" s="28" t="inlineStr">
         <is>
-          <t>— Coverage: —</t>
+          <t>— Coverage: —
+Review action: Document undecidability and administrator/manufacturing trust boundaries; never mark them passed through ordinary testing.</t>
         </is>
       </c>
       <c r="K14" s="28" t="inlineStr">
@@ -2776,10 +2850,14 @@
       </c>
       <c r="L14" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M14" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M14" s="28" t="inlineStr">
+        <is>
+          <t>docs/phase-1/W7-plus-plus-test-objectives.md</t>
+        </is>
+      </c>
       <c r="N14" s="28" t="n"/>
     </row>
     <row r="15" ht="90" customHeight="1" s="14">
@@ -2821,12 +2899,14 @@
       <c r="H15" s="28" t="inlineStr"/>
       <c r="I15" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Limitation/trust-assumption disposition, not an executable acceptance test. Original worksheet claims and statuses retained.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J15" s="28" t="inlineStr">
         <is>
-          <t>— Coverage: Reproducible bitstreams narrow, do not close</t>
+          <t>— Coverage: Reproducible bitstreams narrow, do not close
+Review action: Document undecidability and administrator/manufacturing trust boundaries; never mark them passed through ordinary testing.</t>
         </is>
       </c>
       <c r="K15" s="28" t="inlineStr">
@@ -2836,10 +2916,14 @@
       </c>
       <c r="L15" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M15" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M15" s="28" t="inlineStr">
+        <is>
+          <t>docs/phase-1/W7-plus-plus-test-objectives.md</t>
+        </is>
+      </c>
       <c r="N15" s="28" t="n"/>
     </row>
     <row r="16" ht="90" customHeight="1" s="14">
@@ -2881,12 +2965,14 @@
       <c r="H16" s="28" t="inlineStr"/>
       <c r="I16" s="28" t="inlineStr">
         <is>
-          <t>Original workbook claim, not independently qualified. See original row.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Distribution remains explicitly outside Phase 1.
+Earlier baseline: Original workbook claim, not independently qualified. See original row.</t>
         </is>
       </c>
       <c r="J16" s="28" t="inlineStr">
         <is>
-          <t>— Coverage: —</t>
+          <t>— Coverage: —
+Review action: Keep two-Namespace networking and remote invocation in Phase 2.</t>
         </is>
       </c>
       <c r="K16" s="28" t="inlineStr">
@@ -2896,10 +2982,14 @@
       </c>
       <c r="L16" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M16" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M16" s="28" t="inlineStr">
+        <is>
+          <t>docs/phase-1/W7-plus-plus-test-objectives.md</t>
+        </is>
+      </c>
       <c r="N16" s="28" t="n"/>
     </row>
     <row r="17" ht="90" customHeight="1" s="14">
@@ -4482,7 +4572,7 @@
       </c>
       <c r="F41" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G41" s="28" t="inlineStr">
@@ -4497,10 +4587,16 @@
       </c>
       <c r="I41" s="28" t="inlineStr">
         <is>
-          <t>Defined objective; full acceptance not established by this tracker.</t>
-        </is>
-      </c>
-      <c r="J41" s="28" t="inlineStr"/>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Slot package reports 19 full-core RTL replay tests; CREATE/DESTROY lifecycle evidence includes version-0 issuance, release/reuse at version 1, stale-GT rejection and zeroed reused storage. Private fixture history is explicit.
+Earlier baseline: Defined objective; full acceptance not established by this tracker.</t>
+        </is>
+      </c>
+      <c r="J41" s="28" t="inlineStr">
+        <is>
+          <t>
+Review action: Complete full criterion including retained history, retirement boundaries and live/reused-slot applicability; model evidence is not physical acceptance.</t>
+        </is>
+      </c>
       <c r="K41" s="28" t="inlineStr">
         <is>
           <t>docs/phase-1/04-release/isa-to-fpga-alignment-plan.md</t>
@@ -4508,10 +4604,14 @@
       </c>
       <c r="L41" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M41" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M41" s="28" t="inlineStr">
+        <is>
+          <t>docs/phase-1/mint-slot-package.md; docs/phase-1/mint-destroy-v1-development.md</t>
+        </is>
+      </c>
       <c r="N41" s="28" t="n"/>
     </row>
     <row r="42" ht="90" customHeight="1" s="14">
@@ -4662,7 +4762,7 @@
       </c>
       <c r="F44" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G44" s="28" t="inlineStr">
@@ -4677,12 +4777,14 @@
       </c>
       <c r="I44" s="28" t="inlineStr">
         <is>
-          <t>Defined objective; full acceptance not established by this tracker.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Stronger evidence than the earlier adapted fixtures: 2026-10-20 actual saved NewLayout image, ordinary admission/design paths, authorized Alice 731 round-trip, Mallory NO_CAPABILITY at LOAD PC 1, Alice unchanged. Report records 102 server checks plus JS/image checks. Not rerun in this review.
+Earlier baseline: Defined objective; full acceptance not established by this tracker.</t>
         </is>
       </c>
       <c r="J44" s="28" t="inlineStr">
         <is>
-          <t>Multiple authorized methods read/update one defined record across calls and returns; other records are unchanged; another Thread gains no implicit access; stale allocation references are rejected.</t>
+          <t>Multiple authorized methods read/update one defined record across calls and returns; other records are unchanged; another Thread gains no implicit access; stale allocation references are rejected.
+Review action: Retain exact image/artifact identities and exclusions. Close each full criterion only after its remaining isolation/tuple/lifecycle coverage; no FPGA or power-loss acceptance implied.</t>
         </is>
       </c>
       <c r="K44" s="28" t="inlineStr">
@@ -4692,10 +4794,14 @@
       </c>
       <c r="L44" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M44" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M44" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/saved-alice-mallory-execution.md</t>
+        </is>
+      </c>
       <c r="N44" s="28" t="n"/>
     </row>
     <row r="45" ht="90" customHeight="1" s="14">
@@ -5110,7 +5216,7 @@
       </c>
       <c r="F51" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G51" s="28" t="inlineStr">
@@ -5125,12 +5231,14 @@
       </c>
       <c r="I51" s="28" t="inlineStr">
         <is>
-          <t>Defined objective; full acceptance not established by this tracker.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Saved actor report binds exact image/artifact identities. Named-CALL save reproduction rejects altered code and forged API metadata in isolated tests. This supports integrity/attribution, not full release or field coverage.
+Earlier baseline: Defined objective; full acceptance not established by this tracker.</t>
         </is>
       </c>
       <c r="J51" s="28" t="inlineStr">
         <is>
-          <t>Attach the actual LUMP/configuration and implementation identities to results; hardware claims identify the tested bitstream and board. Mark differences from simulator-only coverage.</t>
+          <t>Attach the actual LUMP/configuration and implementation identities to results; hardware claims identify the tested bitstream and board. Mark differences from simulator-only coverage.
+Review action: Complete item-specific identity/replay coverage and bind exact source, generated image, bitstream and physical observations.</t>
         </is>
       </c>
       <c r="K51" s="28" t="inlineStr">
@@ -5140,12 +5248,12 @@
       </c>
       <c r="L51" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="M51" s="28" t="inlineStr">
         <is>
-          <t>BASE-09: docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/reviews/saved-alice-mallory-execution.md; tests/server/test_named_call_save_attestation.py; BASE-09: docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N51" s="28" t="n"/>
@@ -5577,12 +5685,14 @@
       </c>
       <c r="I58" s="28" t="inlineStr">
         <is>
-          <t>S02 Lambda location jump vs inline JS; S03 continuation/frame/keep-mask differences; no demonstrated internal label X or CR result path</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Native Lambda and compiled Mint/Cleaner CREATE/DESTROY now have bounded simulator/RTL evidence. Historical protected-Mint positive acceptance is explicitly superseded by the CR-preserving Lambda RETURN correction; its cleanup shortcut is not valid authority. Current isolated V1 lifecycle evidence is distinct.
+Earlier baseline: S02 Lambda location jump vs inline JS; S03 continuation/frame/keep-mask differences; no demonstrated internal label X or CR result path</t>
         </is>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>Prefer an existing legal same-artifact X binding plus validated private result-cell LOAD. Otherwise specify smallest architectural change; do not fabricate CRs, make a separate service, or enable old fused opcodes / Engineering trace and same-byte cross-layer tests first. Explicit architectural/provisioning approval if new subobject authority, aliases or continuation semantics are required. Accept exact proposed ABI only after this</t>
+          <t>Prefer an existing legal same-artifact X binding plus validated private result-cell LOAD. Otherwise specify smallest architectural change; do not fabricate CRs, make a separate service, or enable old fused opcodes / Engineering trace and same-byte cross-layer tests first. Explicit architectural/provisioning approval if new subobject authority, aliases or continuation semantics are required. Accept exact proposed ABI only after this
+Review action: Separate native provisioning/result interfaces from historical adapter behavior; complete operational proof/requester/cleanup gates and qualify exact saved service bytes. No live service or board closure.</t>
         </is>
       </c>
       <c r="K58" s="28" t="inlineStr">
@@ -5592,10 +5702,14 @@
       </c>
       <c r="L58" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M58" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M58" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/mint-phase1/native-lambda-binding.md; docs/phase-1/mint-destroy-v1-development.md; docs/reviews/mint-phase1/qualified-protected-namespace.md</t>
+        </is>
+      </c>
       <c r="N58" s="28" t="n"/>
     </row>
     <row r="59" ht="90" customHeight="1" s="14">
@@ -5769,12 +5883,14 @@
       </c>
       <c r="I61" s="28" t="inlineStr">
         <is>
-          <t>S06 per-instruction busy; S07 M6/raw UART/reset and RAM priority; readback alone insufficient</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): CREATE cut-point report records 9 PASS, 2 FAIL, 21 BLOCKED. Seal-only publication checks fail; restored ABA and restart-dependent acceptance remain blocked. This is recorded diagnostic evidence, not a fresh run; harness PASS is not acceptance PASS.
+Earlier baseline: S06 per-instruction busy; S07 M6/raw UART/reset and RAM priority; readback alone insufficient</t>
         </is>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>First prove bounded existing admission/observer exclusion. If impossible, propose minimal interlock/reset containment or explicitly enforceable operational constraints. Prefer no new engine, but never weaken safety to avoid hardware / Engineering reachability and accepted-write latency evidence. Explicit approval for new hardware or restrictions; software gate separate from bitstream milestone</t>
+          <t>First prove bounded existing admission/observer exclusion. If impossible, propose minimal interlock/reset containment or explicitly enforceable operational constraints. Prefer no new engine, but never weaken safety to avoid hardware / Engineering reachability and accepted-write latency evidence. Explicit approval for new hardware or restrictions; software gate separate from bitstream milestone
+Review action: Do not use valid seal as completion oracle. Establish whole-update exclusion, authorized retained-history restart and durable commit independently; no new recovery policy is authorized.</t>
         </is>
       </c>
       <c r="K61" s="28" t="inlineStr">
@@ -5784,10 +5900,14 @@
       </c>
       <c r="L61" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M61" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M61" s="28" t="inlineStr">
+        <is>
+          <t>docs/phase-1/mint-create-cut-points.md; docs/phase-1/mint-destroy-v1-development.md</t>
+        </is>
+      </c>
       <c r="N61" s="28" t="n"/>
     </row>
     <row r="62" ht="90" customHeight="1" s="14">
@@ -5833,12 +5953,14 @@
       </c>
       <c r="I62" s="28" t="inlineStr">
         <is>
-          <t>S10 ordinary transactions/fsync are not a vault; Q54 needs atomic record/pool/counter and trustworthy boot restore</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): CREATE cut-point report records 9 PASS, 2 FAIL, 21 BLOCKED. Seal-only publication checks fail; restored ABA and restart-dependent acceptance remain blocked. This is recorded diagnostic evidence, not a fresh run; harness PASS is not acceptance PASS.
+Earlier baseline: S10 ordinary transactions/fsync are not a vault; Q54 needs atomic record/pool/counter and trustworthy boot restore</t>
         </is>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>Dedicated private transactional store and separate keys; external monotonic revision anchor vs Genesis-verified latest-state procedure. Recommend independent anchor where available / Select custody/backup/latest-state mechanism and actual durability boundary, prove crash cuts and corruption/rollback rejection. No permission to lose pool entries or resume calls</t>
+          <t>Dedicated private transactional store and separate keys; external monotonic revision anchor vs Genesis-verified latest-state procedure. Recommend independent anchor where available / Select custody/backup/latest-state mechanism and actual durability boundary, prove crash cuts and corruption/rollback rejection. No permission to lose pool entries or resume calls
+Review action: Do not use valid seal as completion oracle. Establish whole-update exclusion, authorized retained-history restart and durable commit independently; no new recovery policy is authorized.</t>
         </is>
       </c>
       <c r="K62" s="28" t="inlineStr">
@@ -5848,10 +5970,14 @@
       </c>
       <c r="L62" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M62" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M62" s="28" t="inlineStr">
+        <is>
+          <t>docs/phase-1/mint-create-cut-points.md; docs/phase-1/mint-destroy-v1-development.md</t>
+        </is>
+      </c>
       <c r="N62" s="28" t="n"/>
     </row>
     <row r="63" ht="90" customHeight="1" s="14">
@@ -5961,12 +6087,14 @@
       </c>
       <c r="I64" s="28" t="inlineStr">
         <is>
-          <t>S01 Boot.Namespace role vs S11 Boot.NS seed; Q06 assigned-Owner policy vs legacy Abstract users; free/retired entry representation and virtualGT unresolved</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Native Lambda and compiled Mint/Cleaner CREATE/DESTROY now have bounded simulator/RTL evidence. Historical protected-Mint positive acceptance is explicitly superseded by the CR-preserving Lambda RETURN correction; its cleanup shortcut is not valid authority. Current isolated V1 lifecycle evidence is distinct.
+Earlier baseline: S01 Boot.Namespace role vs S11 Boot.NS seed; Q06 assigned-Owner policy vs legacy Abstract users; free/retired entry representation and virtualGT unresolved</t>
         </is>
       </c>
       <c r="J64" s="28" t="inlineStr">
         <is>
-          <t>Bind Boot to exact approved configuration self-entry, not new name. Configuration-scoped incarnation registry proposed; local T===GT. Reject virtual/non-memory objects until explicit binding exists. Typed validators and retained slot-history records / Engineering exact packing/allocator/zeroing fixtures and resource measurement. Approve identity-lifecycle/compatibility changes and final capacities; do not reopen initial empty targets or change residency</t>
+          <t>Bind Boot to exact approved configuration self-entry, not new name. Configuration-scoped incarnation registry proposed; local T===GT. Reject virtual/non-memory objects until explicit binding exists. Typed validators and retained slot-history records / Engineering exact packing/allocator/zeroing fixtures and resource measurement. Approve identity-lifecycle/compatibility changes and final capacities; do not reopen initial empty targets or change residency
+Review action: Separate native provisioning/result interfaces from historical adapter behavior; complete operational proof/requester/cleanup gates and qualify exact saved service bytes. No live service or board closure.</t>
         </is>
       </c>
       <c r="K64" s="28" t="inlineStr">
@@ -5976,10 +6104,14 @@
       </c>
       <c r="L64" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M64" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M64" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/mint-phase1/native-lambda-binding.md; docs/phase-1/mint-destroy-v1-development.md; docs/reviews/mint-phase1/qualified-protected-namespace.md</t>
+        </is>
+      </c>
       <c r="N64" s="28" t="n"/>
     </row>
     <row r="65" ht="90" customHeight="1" s="14">
@@ -6265,12 +6397,14 @@
       <c r="H69" s="28" t="inlineStr"/>
       <c r="I69" s="28" t="inlineStr">
         <is>
-          <t>Workflow snapshot reports editor-roundtrip failures; root cause/current reproducibility not established.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): 28 October compiler/save work resolves named CALL methods from saved binary APIs; Save's independent recompile now uses trusted lookup too. Prior session recorded five passing isolated save regressions, including altered code, missing target, wrong pin and forged API rejection. Legacy CALL compatibility-test updates are merged, not a fresh full-suite result.
+Earlier baseline: Workflow snapshot reports editor-roundtrip failures; root cause/current reproducibility not established.</t>
         </is>
       </c>
       <c r="J69" s="28" t="inlineStr">
         <is>
-          <t>Reproduce isolated failures; verify create/edit/save, delayed responses, history and draft preservation.</t>
+          <t>Reproduce isolated failures; verify create/edit/save, delayed responses, history and draft preservation.
+Review action: Reconcile remaining item-specific regressions and verify exact saved-source flow. Do not infer complete editor ownership, ISA conformance or release-suite acceptance from focused tests.</t>
         </is>
       </c>
       <c r="K69" s="28" t="inlineStr">
@@ -6280,10 +6414,14 @@
       </c>
       <c r="L69" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M69" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M69" s="28" t="inlineStr">
+        <is>
+          <t>tests/server/test_named_call_save_attestation.py; simulator/test_unresolved_call_compile_error.js; tests/server/test_call_method_lookup_isolated.py</t>
+        </is>
+      </c>
       <c r="N69" s="28" t="n"/>
     </row>
     <row r="70" ht="90" customHeight="1" s="14">
@@ -6513,12 +6651,14 @@
       <c r="H73" s="28" t="inlineStr"/>
       <c r="I73" s="28" t="inlineStr">
         <is>
-          <t>Workflow snapshot flags API-reference and capability-block checks; not freshly reproduced.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): 28 October compiler/save work resolves named CALL methods from saved binary APIs; Save's independent recompile now uses trusted lookup too. Prior session recorded five passing isolated save regressions, including altered code, missing target, wrong pin and forged API rejection. Legacy CALL compatibility-test updates are merged, not a fresh full-suite result.
+Earlier baseline: Workflow snapshot flags API-reference and capability-block checks; not freshly reproduced.</t>
         </is>
       </c>
       <c r="J73" s="28" t="inlineStr">
         <is>
-          <t>Reconcile approved ISA, compiler forms, reference search and examples; retain explicit historical distinctions.</t>
+          <t>Reconcile approved ISA, compiler forms, reference search and examples; retain explicit historical distinctions.
+Review action: Reconcile remaining item-specific regressions and verify exact saved-source flow. Do not infer complete editor ownership, ISA conformance or release-suite acceptance from focused tests.</t>
         </is>
       </c>
       <c r="K73" s="28" t="inlineStr">
@@ -6528,12 +6668,12 @@
       </c>
       <c r="L73" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="M73" s="28" t="inlineStr">
         <is>
-          <t>BASE-08: docs/reviews/phase1-baseline/README.md</t>
+          <t>tests/server/test_named_call_save_attestation.py; simulator/test_unresolved_call_compile_error.js; tests/server/test_call_method_lookup_isolated.py; BASE-08: docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N73" s="28" t="n"/>
@@ -6645,12 +6785,14 @@
       </c>
       <c r="I75" s="28" t="inlineStr">
         <is>
-          <t>G1 finds entry/continuation mismatch and unproven result authority.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Native Lambda and compiled Mint/Cleaner CREATE/DESTROY now have bounded simulator/RTL evidence. Historical protected-Mint positive acceptance is explicitly superseded by the CR-preserving Lambda RETURN correction; its cleanup shortcut is not valid authority. Current isolated V1 lifecycle evidence is distinct.
+Earlier baseline: G1 finds entry/continuation mismatch and unproven result authority.</t>
         </is>
       </c>
       <c r="J75" s="28" t="inlineStr">
         <is>
-          <t>Resolve ISA contract; prove legal binding and result LOAD through real gates.</t>
+          <t>Resolve ISA contract; prove legal binding and result LOAD through real gates.
+Review action: Separate native provisioning/result interfaces from historical adapter behavior; complete operational proof/requester/cleanup gates and qualify exact saved service bytes. No live service or board closure.</t>
         </is>
       </c>
       <c r="K75" s="28" t="inlineStr">
@@ -6660,10 +6802,14 @@
       </c>
       <c r="L75" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M75" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M75" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/mint-phase1/native-lambda-binding.md; docs/phase-1/mint-destroy-v1-development.md; docs/reviews/mint-phase1/qualified-protected-namespace.md</t>
+        </is>
+      </c>
       <c r="N75" s="28" t="n"/>
     </row>
     <row r="76" ht="90" customHeight="1" s="14">
@@ -7065,12 +7211,14 @@
       <c r="H82" s="28" t="inlineStr"/>
       <c r="I82" s="28" t="inlineStr">
         <is>
-          <t>Exact-byte checks retained independently of catalog status; pending bytes, changed files and immutable local derivatives tested. Full seal/replay/field coverage not established.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Saved actor report binds exact image/artifact identities. Named-CALL save reproduction rejects altered code and forged API metadata in isolated tests. This supports integrity/attribution, not full release or field coverage.
+Earlier baseline: Exact-byte checks retained independently of catalog status; pending bytes, changed files and immutable local derivatives tested. Full seal/replay/field coverage not established.</t>
         </is>
       </c>
       <c r="J82" s="28" t="inlineStr">
         <is>
-          <t>Reject tampering, stale/replayed seals and mismatched artifact/slot/generation; prove every covered field and permitted F/G mutation.</t>
+          <t>Reject tampering, stale/replayed seals and mismatched artifact/slot/generation; prove every covered field and permitted F/G mutation.
+Review action: Complete item-specific identity/replay coverage and bind exact source, generated image, bitstream and physical observations.</t>
         </is>
       </c>
       <c r="K82" s="28" t="inlineStr">
@@ -7080,12 +7228,12 @@
       </c>
       <c r="L82" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="M82" s="28" t="inlineStr">
         <is>
-          <t>BASE-03: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md</t>
+          <t>docs/reviews/saved-alice-mallory-execution.md; tests/server/test_named_call_save_attestation.py; BASE-03: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md</t>
         </is>
       </c>
       <c r="N82" s="28" t="n"/>
@@ -7129,12 +7277,14 @@
       <c r="H83" s="28" t="inlineStr"/>
       <c r="I83" s="28" t="inlineStr">
         <is>
-          <t>A successful checksum comparison does not prove exclusion or durable commit.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): CREATE cut-point report records 9 PASS, 2 FAIL, 21 BLOCKED. Seal-only publication checks fail; restored ABA and restart-dependent acceptance remain blocked. This is recorded diagnostic evidence, not a fresh run; harness PASS is not acceptance PASS.
+Earlier baseline: A successful checksum comparison does not prove exclusion or durable commit.</t>
         </is>
       </c>
       <c r="J83" s="28" t="inlineStr">
         <is>
-          <t>Inject interruptions between data/seal writes; no partial or stale authority usable after reset; no implicit retry/rollback.</t>
+          <t>Inject interruptions between data/seal writes; no partial or stale authority usable after reset; no implicit retry/rollback.
+Review action: Do not use valid seal as completion oracle. Establish whole-update exclusion, authorized retained-history restart and durable commit independently; no new recovery policy is authorized.</t>
         </is>
       </c>
       <c r="K83" s="28" t="inlineStr">
@@ -7144,10 +7294,14 @@
       </c>
       <c r="L83" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M83" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M83" s="28" t="inlineStr">
+        <is>
+          <t>docs/phase-1/mint-create-cut-points.md; docs/phase-1/mint-destroy-v1-development.md</t>
+        </is>
+      </c>
       <c r="N83" s="28" t="n"/>
     </row>
     <row r="84" ht="90" customHeight="1" s="14">
@@ -7313,12 +7467,14 @@
       <c r="H86" s="28" t="inlineStr"/>
       <c r="I86" s="28" t="inlineStr">
         <is>
-          <t>Assembler workflow reports failure; simulator agreement alone is not an independent oracle.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): 28 October compiler/save work resolves named CALL methods from saved binary APIs; Save's independent recompile now uses trusted lookup too. Prior session recorded five passing isolated save regressions, including altered code, missing target, wrong pin and forged API rejection. Legacy CALL compatibility-test updates are merged, not a fresh full-suite result.
+Earlier baseline: Assembler workflow reports failure; simulator agreement alone is not an independent oracle.</t>
         </is>
       </c>
       <c r="J86" s="28" t="inlineStr">
         <is>
-          <t>Use hand-encoded vectors for all forms, bounds, conditions, retired encodings and CR13 restrictions.</t>
+          <t>Use hand-encoded vectors for all forms, bounds, conditions, retired encodings and CR13 restrictions.
+Review action: Reconcile remaining item-specific regressions and verify exact saved-source flow. Do not infer complete editor ownership, ISA conformance or release-suite acceptance from focused tests.</t>
         </is>
       </c>
       <c r="K86" s="28" t="inlineStr">
@@ -7328,12 +7484,12 @@
       </c>
       <c r="L86" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="M86" s="28" t="inlineStr">
         <is>
-          <t>BASE-01: docs/reviews/phase1-baseline/README.md; BASE-03: docs/reviews/phase1-baseline/README.md</t>
+          <t>tests/server/test_named_call_save_attestation.py; simulator/test_unresolved_call_compile_error.js; tests/server/test_call_method_lookup_isolated.py; BASE-01: docs/reviews/phase1-baseline/README.md; BASE-03: docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N86" s="28" t="n"/>
@@ -7565,12 +7721,14 @@
       <c r="H90" s="28" t="inlineStr"/>
       <c r="I90" s="28" t="inlineStr">
         <is>
-          <t>Alice/Mallory fixtures adapt old code in isolated RAM; originals remain immutable.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Stronger evidence than the earlier adapted fixtures: 2026-10-20 actual saved NewLayout image, ordinary admission/design paths, authorized Alice 731 round-trip, Mallory NO_CAPABILITY at LOAD PC 1, Alice unchanged. Report records 102 server checks plus JS/image checks. Not rerun in this review.
+Earlier baseline: Alice/Mallory fixtures adapt old code in isolated RAM; originals remain immutable.</t>
         </is>
       </c>
       <c r="J90" s="28" t="inlineStr">
         <is>
-          <t>Record exact original/adapted words and current ISA; never claim adapted runs qualify historical binary unchanged.</t>
+          <t>Record exact original/adapted words and current ISA; never claim adapted runs qualify historical binary unchanged.
+Review action: Retain exact image/artifact identities and exclusions. Close each full criterion only after its remaining isolation/tuple/lifecycle coverage; no FPGA or power-loss acceptance implied.</t>
         </is>
       </c>
       <c r="K90" s="28" t="inlineStr">
@@ -7580,12 +7738,12 @@
       </c>
       <c r="L90" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="M90" s="28" t="inlineStr">
         <is>
-          <t>BASE-07: docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/reviews/saved-alice-mallory-execution.md; BASE-07: docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N90" s="28" t="n"/>
@@ -7629,12 +7787,14 @@
       <c r="H91" s="28" t="inlineStr"/>
       <c r="I91" s="28" t="inlineStr">
         <is>
-          <t>Prior inspection found 22/39 recorded build inputs differ; this is not a new build verification.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Reviewed software and RTL reports explicitly exclude physical-board qualification. No new exact-build or board acceptance run was performed for this update.
+Earlier baseline: Prior inspection found 22/39 recorded build inputs differ; this is not a new build verification.</t>
         </is>
       </c>
       <c r="J91" s="28" t="inlineStr">
         <is>
-          <t>Regenerate authorized exact inputs; verify hashes, ROM/configuration, timing, DRC and artifact sidecars.</t>
+          <t>Regenerate authorized exact inputs; verify hashes, ROM/configuration, timing, DRC and artifact sidecars.
+Review action: Freeze the approved candidate and obtain matching build/timing/provenance plus separately authorized physical acceptance. Never relabel historical bitstreams.</t>
         </is>
       </c>
       <c r="K91" s="28" t="inlineStr">
@@ -7644,12 +7804,12 @@
       </c>
       <c r="L91" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="M91" s="28" t="inlineStr">
         <is>
-          <t>BASE-06: docs/reviews/phase1-baseline/README.md; BASE-09: docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/W7-plus-plus-test-objectives.md; docs/phase-1/mint-destroy-v1-development.md; BASE-06: docs/reviews/phase1-baseline/README.md; BASE-09: docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N91" s="28" t="n"/>
@@ -7697,12 +7857,14 @@
       </c>
       <c r="I92" s="28" t="inlineStr">
         <is>
-          <t>No physical Phase 1 acceptance performed for this tracker.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Reviewed software and RTL reports explicitly exclude physical-board qualification. No new exact-build or board acceptance run was performed for this update.
+Earlier baseline: No physical Phase 1 acceptance performed for this tracker.</t>
         </is>
       </c>
       <c r="J92" s="28" t="inlineStr">
         <is>
-          <t>After separate authorization, run H19/H20 with exact board/build identity and retained raw observations.</t>
+          <t>After separate authorization, run H19/H20 with exact board/build identity and retained raw observations.
+Review action: Freeze the approved candidate and obtain matching build/timing/provenance plus separately authorized physical acceptance. Never relabel historical bitstreams.</t>
         </is>
       </c>
       <c r="K92" s="28" t="inlineStr">
@@ -7712,12 +7874,12 @@
       </c>
       <c r="L92" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="M92" s="28" t="inlineStr">
         <is>
-          <t>BASE-09: docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/W7-plus-plus-test-objectives.md; docs/phase-1/mint-destroy-v1-development.md; BASE-09: docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N92" s="28" t="n"/>
@@ -7761,12 +7923,14 @@
       <c r="H93" s="28" t="inlineStr"/>
       <c r="I93" s="28" t="inlineStr">
         <is>
-          <t>Fresh combined merge verification: 190 passed, 2 failed; no skips/xfails. Admission/allocation/private simulation: 128 passes. Independent image suite: 62 passes, 2 migration failures (parent/explicit config). Historical migration copies device address 0x40000014 into resident NS[10]; generator correctly rejects out-of-RAM placement. Other regression groups remain open.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): 28 October compiler/save work resolves named CALL methods from saved binary APIs; Save's independent recompile now uses trusted lookup too. Prior session recorded five passing isolated save regressions, including altered code, missing target, wrong pin and forged API rejection. Legacy CALL compatibility-test updates are merged, not a fresh full-suite result.
+Earlier baseline: Fresh combined merge verification: 190 passed, 2 failed; no skips/xfails. Admission/allocation/private simulation: 128 passes. Independent image suite: 62 passes, 2 migration failures (parent/explicit config). Historical migration copies device address 0x40000014 into resident NS[10]; generator correctly rejects out-of-RAM placement. Other regression groups remain open.</t>
         </is>
       </c>
       <c r="J93" s="28" t="inlineStr">
         <is>
-          <t>Isolate current failures, classify stale fixtures versus defects; record commands, output, identities and reruns.</t>
+          <t>Isolate current failures, classify stale fixtures versus defects; record commands, output, identities and reruns.
+Review action: Reconcile remaining item-specific regressions and verify exact saved-source flow. Do not infer complete editor ownership, ISA conformance or release-suite acceptance from focused tests.</t>
         </is>
       </c>
       <c r="K93" s="28" t="inlineStr">
@@ -7776,12 +7940,12 @@
       </c>
       <c r="L93" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="M93" s="28" t="inlineStr">
         <is>
-          <t>BASE-01: docs/reviews/phase1-baseline/README.md; BASE-03: docs/reviews/phase1-baseline/README.md; BASE-08: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md; docs/reviews/phase1-baseline/namespace-authority-progress.md#combined-post-merge-verification--17-october-2026</t>
+          <t>tests/server/test_named_call_save_attestation.py; simulator/test_unresolved_call_compile_error.js; tests/server/test_call_method_lookup_isolated.py; BASE-01: docs/reviews/phase1-baseline/README.md; BASE-03: docs/reviews/phase1-baseline/README.md; BASE-08: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md; docs/reviews/phase1-baseline/namespace-authority-progress.md#combined-post-merge-verification--17-october-2026</t>
         </is>
       </c>
       <c r="N93" s="28" t="n"/>
@@ -8261,12 +8425,14 @@
       </c>
       <c r="I101" s="28" t="inlineStr">
         <is>
-          <t>57-answer ledger and Genesis review established; G1-G8 open. First credential Create-only in Boot, with permanently empty Replace/Destroy targets. Absent from inspected saved Namespace.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Native Lambda and compiled Mint/Cleaner CREATE/DESTROY now have bounded simulator/RTL evidence. Historical protected-Mint positive acceptance is explicitly superseded by the CR-preserving Lambda RETURN correction; its cleanup shortcut is not valid authority. Current isolated V1 lifecycle evidence is distinct.
+Earlier baseline: 57-answer ledger and Genesis review established; G1-G8 open. First credential Create-only in Boot, with permanently empty Replace/Destroy targets. Absent from inspected saved Namespace.</t>
         </is>
       </c>
       <c r="J101" s="28" t="inlineStr">
         <is>
-          <t>Record exact artifact, approved destination/binding, resident footprint and simulator/RTL/board acceptance separately.</t>
+          <t>Record exact artifact, approved destination/binding, resident footprint and simulator/RTL/board acceptance separately.
+Review action: Separate native provisioning/result interfaces from historical adapter behavior; complete operational proof/requester/cleanup gates and qualify exact saved service bytes. No live service or board closure.</t>
         </is>
       </c>
       <c r="K101" s="28" t="inlineStr">
@@ -8276,10 +8442,14 @@
       </c>
       <c r="L101" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M101" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M101" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/mint-phase1/native-lambda-binding.md; docs/phase-1/mint-destroy-v1-development.md; docs/reviews/mint-phase1/qualified-protected-namespace.md</t>
+        </is>
+      </c>
       <c r="N101" s="28" t="n"/>
     </row>
     <row r="102" ht="90" customHeight="1" s="14">
@@ -8445,12 +8615,14 @@
       <c r="H104" s="28" t="inlineStr"/>
       <c r="I104" s="28" t="inlineStr">
         <is>
-          <t>Merged isolated simulator fixtures cover own-tuple DWRITE/DREAD and adapted legacy scenarios; not a new run or board acceptance. Not a saved resident here.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Stronger evidence than the earlier adapted fixtures: 2026-10-20 actual saved NewLayout image, ordinary admission/design paths, authorized Alice 731 round-trip, Mallory NO_CAPABILITY at LOAD PC 1, Alice unchanged. Report records 102 server checks plus JS/image checks. Not rerun in this review.
+Earlier baseline: Merged isolated simulator fixtures cover own-tuple DWRITE/DREAD and adapted legacy scenarios; not a new run or board acceptance. Not a saved resident here.</t>
         </is>
       </c>
       <c r="J104" s="28" t="inlineStr">
         <is>
-          <t>Record exact artifact, approved destination/binding, resident footprint and simulator/RTL/board acceptance separately.</t>
+          <t>Record exact artifact, approved destination/binding, resident footprint and simulator/RTL/board acceptance separately.
+Review action: Retain exact image/artifact identities and exclusions. Close each full criterion only after its remaining isolation/tuple/lifecycle coverage; no FPGA or power-loss acceptance implied.</t>
         </is>
       </c>
       <c r="K104" s="28" t="inlineStr">
@@ -8460,10 +8632,14 @@
       </c>
       <c r="L104" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M104" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M104" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/saved-alice-mallory-execution.md</t>
+        </is>
+      </c>
       <c r="N104" s="28" t="n"/>
     </row>
     <row r="105" ht="90" customHeight="1" s="14">
@@ -8505,12 +8681,14 @@
       <c r="H105" s="28" t="inlineStr"/>
       <c r="I105" s="28" t="inlineStr">
         <is>
-          <t>Merged seven tuple scenarios include absent-capability denial, own-tuple positive control, foreign/range read/write denial and full 58-word Alice integrity. No new run or board proof.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Stronger evidence than the earlier adapted fixtures: 2026-10-20 actual saved NewLayout image, ordinary admission/design paths, authorized Alice 731 round-trip, Mallory NO_CAPABILITY at LOAD PC 1, Alice unchanged. Report records 102 server checks plus JS/image checks. Not rerun in this review.
+Earlier baseline: Merged seven tuple scenarios include absent-capability denial, own-tuple positive control, foreign/range read/write denial and full 58-word Alice integrity. No new run or board proof.</t>
         </is>
       </c>
       <c r="J105" s="28" t="inlineStr">
         <is>
-          <t>Record exact artifact, approved destination/binding, resident footprint and simulator/RTL/board acceptance separately.</t>
+          <t>Record exact artifact, approved destination/binding, resident footprint and simulator/RTL/board acceptance separately.
+Review action: Retain exact image/artifact identities and exclusions. Close each full criterion only after its remaining isolation/tuple/lifecycle coverage; no FPGA or power-loss acceptance implied.</t>
         </is>
       </c>
       <c r="K105" s="28" t="inlineStr">
@@ -8520,10 +8698,14 @@
       </c>
       <c r="L105" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M105" s="28" t="n"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="M105" s="28" t="inlineStr">
+        <is>
+          <t>docs/reviews/saved-alice-mallory-execution.md</t>
+        </is>
+      </c>
       <c r="N105" s="28" t="n"/>
     </row>
     <row r="106" ht="100" customHeight="1" s="14">
@@ -8569,12 +8751,14 @@
       </c>
       <c r="I106" s="28" t="inlineStr">
         <is>
-          <t>Confirmed dependency-initialization failure; not an ISA verdict. Existing assembler workflow throws TypeError: ChurchAssembler is not a constructor at compiler line 220. Fresh in-memory probe reproduces it with global assembler undefined; injecting the real constructor removes this exception (the sample still has one compile diagnostic).</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): 28 October compiler/save work resolves named CALL methods from saved binary APIs; Save's independent recompile now uses trusted lookup too. Prior session recorded five passing isolated save regressions, including altered code, missing target, wrong pin and forged API rejection. Legacy CALL compatibility-test updates are merged, not a fresh full-suite result.
+Earlier baseline: Confirmed dependency-initialization failure; not an ISA verdict. Existing assembler workflow throws TypeError: ChurchAssembler is not a constructor at compiler line 220. Fresh in-memory probe reproduces it with global assembler undefined; injecting the real constructor removes this exception (the sample still has one compile diagnostic).</t>
         </is>
       </c>
       <c r="J106" s="28" t="inlineStr">
         <is>
-          <t>Establish explicit Node/compiler dependency setup and regression coverage; rerun isolated assembler suite before interpreting encoding failures. Do not weaken retired-opcode diagnostics.</t>
+          <t>Establish explicit Node/compiler dependency setup and regression coverage; rerun isolated assembler suite before interpreting encoding failures. Do not weaken retired-opcode diagnostics.
+Review action: Reconcile remaining item-specific regressions and verify exact saved-source flow. Do not infer complete editor ownership, ISA conformance or release-suite acceptance from focused tests.</t>
         </is>
       </c>
       <c r="K106" s="28" t="inlineStr">
@@ -8584,12 +8768,12 @@
       </c>
       <c r="L106" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="M106" s="28" t="inlineStr">
         <is>
-          <t>docs/reviews/phase1-baseline/README.md</t>
+          <t>tests/server/test_named_call_save_attestation.py; simulator/test_unresolved_call_compile_error.js; tests/server/test_call_method_lookup_isolated.py; docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N106" s="28" t="n"/>
@@ -9045,12 +9229,14 @@
       </c>
       <c r="I113" s="28" t="inlineStr">
         <is>
-          <t>Probable fixture/contract drift; not a fresh test result. Existing run fails in test_abs_saved_api.js: compiled method declarations unavailable. The fixture invokes _formatLumpApiDefinition('LED', []); failure occurs before the advertised reference comparison completes.</t>
+          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): 28 October compiler/save work resolves named CALL methods from saved binary APIs; Save's independent recompile now uses trusted lookup too. Prior session recorded five passing isolated save regressions, including altered code, missing target, wrong pin and forged API rejection. Legacy CALL compatibility-test updates are merged, not a fresh full-suite result.
+Earlier baseline: Probable fixture/contract drift; not a fresh test result. Existing run fails in test_abs_saved_api.js: compiled method declarations unavailable. The fixture invokes _formatLumpApiDefinition('LED', []); failure occurs before the advertised reference comparison completes.</t>
         </is>
       </c>
       <c r="J113" s="28" t="inlineStr">
         <is>
-          <t>Supply authentic compiled metadata in the fixture, or establish why valid metadata is lost; retain fail-closed refusal to infer API from another LUMP.</t>
+          <t>Supply authentic compiled metadata in the fixture, or establish why valid metadata is lost; retain fail-closed refusal to infer API from another LUMP.
+Review action: Reconcile remaining item-specific regressions and verify exact saved-source flow. Do not infer complete editor ownership, ISA conformance or release-suite acceptance from focused tests.</t>
         </is>
       </c>
       <c r="K113" s="28" t="inlineStr">
@@ -9060,12 +9246,12 @@
       </c>
       <c r="L113" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="M113" s="28" t="inlineStr">
         <is>
-          <t>docs/reviews/phase1-baseline/README.md</t>
+          <t>tests/server/test_named_call_save_attestation.py; simulator/test_unresolved_call_compile_error.js; tests/server/test_call_method_lookup_isolated.py; docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N113" s="28" t="n"/>
@@ -9162,10 +9348,49 @@
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="M2" r:id="review20261028_2"/>
+    <hyperlink ref="M3" r:id="review20261028_3"/>
+    <hyperlink ref="M4" r:id="review20261028_4"/>
+    <hyperlink ref="M5" r:id="review20261028_5"/>
+    <hyperlink ref="M6" r:id="review20261028_6"/>
+    <hyperlink ref="M7" r:id="review20261028_7"/>
+    <hyperlink ref="M8" r:id="review20261028_8"/>
+    <hyperlink ref="M9" r:id="review20261028_9"/>
+    <hyperlink ref="M10" r:id="review20261028_10"/>
+    <hyperlink ref="M11" r:id="review20261028_11"/>
+    <hyperlink ref="M12" r:id="review20261028_12"/>
+    <hyperlink ref="M13" r:id="review20261028_13"/>
+    <hyperlink ref="M14" r:id="review20261028_14"/>
+    <hyperlink ref="M15" r:id="review20261028_15"/>
+    <hyperlink ref="M16" r:id="review20261028_16"/>
+    <hyperlink ref="M104" r:id="review20261028_104"/>
+    <hyperlink ref="M105" r:id="review20261028_105"/>
+    <hyperlink ref="M90" r:id="review20261028_90"/>
+    <hyperlink ref="M44" r:id="review20261028_44"/>
+    <hyperlink ref="M69" r:id="review20261028_69"/>
+    <hyperlink ref="M73" r:id="review20261028_73"/>
+    <hyperlink ref="M86" r:id="review20261028_86"/>
+    <hyperlink ref="M93" r:id="review20261028_93"/>
+    <hyperlink ref="M106" r:id="review20261028_106"/>
+    <hyperlink ref="M113" r:id="review20261028_113"/>
+    <hyperlink ref="M101" r:id="review20261028_101"/>
+    <hyperlink ref="M58" r:id="review20261028_58"/>
+    <hyperlink ref="M64" r:id="review20261028_64"/>
+    <hyperlink ref="M75" r:id="review20261028_75"/>
+    <hyperlink ref="M61" r:id="review20261028_61"/>
+    <hyperlink ref="M62" r:id="review20261028_62"/>
+    <hyperlink ref="M83" r:id="review20261028_83"/>
+    <hyperlink ref="M41" r:id="review20261028_41"/>
+    <hyperlink ref="M82" r:id="review20261028_82"/>
+    <hyperlink ref="M51" r:id="review20261028_51"/>
+    <hyperlink ref="M91" r:id="review20261028_91"/>
+    <hyperlink ref="M92" r:id="review20261028_92"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -9207,7 +9432,7 @@
       </c>
       <c r="B2" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C2" s="28" t="n"/>
@@ -9260,7 +9485,7 @@
       </c>
       <c r="B6" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Not run")</f>
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="C6" s="28" t="n"/>
       <c r="D6" s="28" t="n"/>
@@ -9273,7 +9498,7 @@
       </c>
       <c r="B7" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Needs verification")</f>
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="C7" s="28" t="n"/>
       <c r="D7" s="28" t="n"/>
@@ -9735,7 +9960,7 @@
       </c>
       <c r="B6" s="28" t="inlineStr">
         <is>
-          <t>Open: work or decision remains. Blocked: prerequisite authority, contract or mechanism missing. Not run: defined objective with no qualifying run recorded.</t>
+          <t>Open: work/decision remains. Blocked: prerequisite missing. Not run: no qualifying objective run. Needs verification may include partial simulator/RTL evidence; it is not a threat pass. Limitations retain their original disposition.</t>
         </is>
       </c>
     </row>
@@ -9747,7 +9972,7 @@
       </c>
       <c r="B7" s="28" t="inlineStr">
         <is>
-          <t>No new simulator, RTL or hardware runs were performed to populate this workbook; workflow snapshot failures are leads, not confirmed current defects.</t>
+          <t>28 October update reviews recorded reports and prior-session focused tests; no fresh acceptance run. Threat Map, Summary and Method remain byte-for-byte unchanged. No W7 threat newly passed. Hardware, W7 baseline and full coverage remain separate gates.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update threat test plan and add validation automation scripts
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
+++ b/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
@@ -4196,7 +4196,7 @@
       </c>
       <c r="F35" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G35" s="28" t="inlineStr">
@@ -4211,12 +4211,14 @@
       </c>
       <c r="I35" s="28" t="inlineStr">
         <is>
-          <t>Defined objective; full acceptance not established by this tracker.</t>
+          <t>Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0. Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery.
+Earlier evidence: Defined objective; full acceptance not established by this tracker.</t>
         </is>
       </c>
       <c r="J35" s="28" t="inlineStr">
         <is>
-          <t>Compare committed registers/flags/memory/faults, not internal cycle counts except deadline/completion bounds. No forced X values or stale model accepted.</t>
+          <t>Combined-candidate next action (2026-10-29): Complete same-fixture cross-layer state comparison and separately authorized physical replay; boot-only vendor evidence does not establish mapped recovery.
+Original criterion / prior actions: Compare committed registers/flags/memory/faults, not internal cycle counts except deadline/completion bounds. No forced X values or stale model accepted.</t>
         </is>
       </c>
       <c r="K35" s="28" t="inlineStr">
@@ -4226,12 +4228,12 @@
       </c>
       <c r="L35" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="M35" s="28" t="inlineStr">
         <is>
-          <t>BASE-06: docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; BASE-06: docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N35" s="28" t="n"/>
@@ -4264,7 +4266,7 @@
       </c>
       <c r="F36" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G36" s="28" t="inlineStr">
@@ -4279,12 +4281,14 @@
       </c>
       <c r="I36" s="28" t="inlineStr">
         <is>
-          <t>Defined objective; full acceptance not established by this tracker.</t>
+          <t>Update 2026-10-29 — combined candidate: Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery. Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0.
+Earlier evidence: Defined objective; full acceptance not established by this tracker.</t>
         </is>
       </c>
       <c r="J36" s="28" t="inlineStr">
         <is>
-          <t>Repeatable outcomes tied to bundle/input hashes, board identity, clock, logs and observed completion; no prior-run telemetry counted as new evidence.</t>
+          <t>Combined-candidate next action (2026-10-29): Perform exact combined-build cold/warm boots, repeated handoffs and physical recovery after separate programming approval.
+Original criterion / prior actions: Repeatable outcomes tied to bundle/input hashes, board identity, clock, logs and observed completion; no prior-run telemetry counted as new evidence.</t>
         </is>
       </c>
       <c r="K36" s="28" t="inlineStr">
@@ -4294,12 +4298,12 @@
       </c>
       <c r="L36" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="M36" s="28" t="inlineStr">
         <is>
-          <t>BASE-06: docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; BASE-06: docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N36" s="28" t="n"/>
@@ -5231,13 +5235,15 @@
       </c>
       <c r="I51" s="28" t="inlineStr">
         <is>
-          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Saved actor report binds exact image/artifact identities. Named-CALL save reproduction rejects altered code and forged API metadata in isolated tests. This supports integrity/attribution, not full release or field coverage.
+          <t>Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0. Build IN PROGRESS as last reported: Vivado 2026.1 opened the validated checkpoint on 2026-10-29 at 18:13:31 (tool-reported time). No completed routing/timing/DRC result or combined BIT yet reported. No combined board programming.
+Earlier evidence: Review 2026-10-28 (recorded evidence; no fresh acceptance run): Saved actor report binds exact image/artifact identities. Named-CALL save reproduction rejects altered code and forged API metadata in isolated tests. This supports integrity/attribution, not full release or field coverage.
 Earlier baseline: Defined objective; full acceptance not established by this tracker.</t>
         </is>
       </c>
       <c r="J51" s="28" t="inlineStr">
         <is>
-          <t>Attach the actual LUMP/configuration and implementation identities to results; hardware claims identify the tested bitstream and board. Mark differences from simulator-only coverage.
+          <t>Combined-candidate next action (2026-10-29): Retain image/source/checkpoint/evidence hashes, then bind the routed BIT receipt and physical observations; do not relabel the earlier BIT.
+Original criterion / prior actions: Attach the actual LUMP/configuration and implementation identities to results; hardware claims identify the tested bitstream and board. Mark differences from simulator-only coverage.
 Review action: Complete item-specific identity/replay coverage and bind exact source, generated image, bitstream and physical observations.</t>
         </is>
       </c>
@@ -5248,12 +5254,12 @@
       </c>
       <c r="L51" s="28" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="M51" s="28" t="inlineStr">
         <is>
-          <t>docs/reviews/saved-alice-mallory-execution.md; tests/server/test_named_call_save_attestation.py; BASE-09: docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; docs/reviews/saved-alice-mallory-execution.md; tests/server/test_named_call_save_attestation.py; BASE-09: docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N51" s="28" t="n"/>
@@ -7597,12 +7603,14 @@
       <c r="H88" s="28" t="inlineStr"/>
       <c r="I88" s="28" t="inlineStr">
         <is>
-          <t>Fresh combined verification: resident addresses 1024/7872, complete body identity, Thread ranges, matching Step-2 placements and private simulation checks pass without xfail exemptions. This is image-generator evidence only; same-byte simulator/RTL instruction conformance remains unverified.</t>
+          <t>Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0. Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery.
+Earlier evidence: Fresh combined verification: resident addresses 1024/7872, complete body identity, Thread ranges, matching Step-2 placements and private simulation checks pass without xfail exemptions. This is image-generator evidence only; same-byte simulator/RTL instruction conformance remains unverified.</t>
         </is>
       </c>
       <c r="J88" s="28" t="inlineStr">
         <is>
-          <t>Compare current ISA and simulator/RTL using immutable fixture identities and exact initial state.</t>
+          <t>Combined-candidate next action (2026-10-29): Retain this exact-image result without claiming full CHANGE/SWITCH or all-profile conformance.
+Original criterion / prior actions: Compare current ISA and simulator/RTL using immutable fixture identities and exact initial state.</t>
         </is>
       </c>
       <c r="K88" s="28" t="inlineStr">
@@ -7612,12 +7620,12 @@
       </c>
       <c r="L88" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="M88" s="28" t="inlineStr">
         <is>
-          <t>BASE-04: docs/reviews/phase1-baseline/README.md; BASE-05: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md#combined-post-merge-verification--17-october-2026</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; BASE-04: docs/reviews/phase1-baseline/README.md; BASE-05: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md#combined-post-merge-verification--17-october-2026</t>
         </is>
       </c>
       <c r="N88" s="28" t="n"/>
@@ -7661,12 +7669,14 @@
       <c r="H89" s="28" t="inlineStr"/>
       <c r="I89" s="28" t="inlineStr">
         <is>
-          <t>Elapsed board clocks cannot be inferred from browser step speed.</t>
+          <t>Update 2026-10-29 — combined candidate: Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery.
+Earlier evidence: Elapsed board clocks cannot be inferred from browser step speed.</t>
         </is>
       </c>
       <c r="J89" s="28" t="inlineStr">
         <is>
-          <t>Validate fault precedence and pre-recovery state; separate logical simulator checks from timed RTL/board proof.</t>
+          <t>Combined-candidate next action (2026-10-29): Verify remaining first-fault/precedence and physical timing objectives; model bounds are not FPGA elapsed-time measurements.
+Original criterion / prior actions: Validate fault precedence and pre-recovery state; separate logical simulator checks from timed RTL/board proof.</t>
         </is>
       </c>
       <c r="K89" s="28" t="inlineStr">
@@ -7676,10 +7686,14 @@
       </c>
       <c r="L89" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M89" s="28" t="n"/>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="M89" s="28" t="inlineStr">
+        <is>
+          <t>docs/phase-1/combined-validation-status-20261029.md</t>
+        </is>
+      </c>
       <c r="N89" s="28" t="n"/>
     </row>
     <row r="90" ht="90" customHeight="1" s="14">
@@ -7776,7 +7790,7 @@
       </c>
       <c r="F91" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G91" s="28" t="inlineStr">
@@ -7787,13 +7801,15 @@
       <c r="H91" s="28" t="inlineStr"/>
       <c r="I91" s="28" t="inlineStr">
         <is>
-          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Reviewed software and RTL reports explicitly exclude physical-board qualification. No new exact-build or board acceptance run was performed for this update.
+          <t>Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0. Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery. Build IN PROGRESS as last reported: Vivado 2026.1 opened the validated checkpoint on 2026-10-29 at 18:13:31 (tool-reported time). No completed routing/timing/DRC result or combined BIT yet reported. No combined board programming.
+Earlier evidence: Review 2026-10-28 (recorded evidence; no fresh acceptance run): Reviewed software and RTL reports explicitly exclude physical-board qualification. No new exact-build or board acceptance run was performed for this update.
 Earlier baseline: Prior inspection found 22/39 recorded build inputs differ; this is not a new build verification.</t>
         </is>
       </c>
       <c r="J91" s="28" t="inlineStr">
         <is>
-          <t>Regenerate authorized exact inputs; verify hashes, ROM/configuration, timing, DRC and artifact sidecars.
+          <t>Combined-candidate next action (2026-10-29): Review COMBINED_IMPLEMENTATION_PASS, exit 0, timing/DRC reports and hash-bearing receipt before accepting the experimental build.
+Original criterion / prior actions: Regenerate authorized exact inputs; verify hashes, ROM/configuration, timing, DRC and artifact sidecars.
 Review action: Freeze the approved candidate and obtain matching build/timing/provenance plus separately authorized physical acceptance. Never relabel historical bitstreams.</t>
         </is>
       </c>
@@ -7804,12 +7820,12 @@
       </c>
       <c r="L91" s="28" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="M91" s="28" t="inlineStr">
         <is>
-          <t>docs/phase-1/W7-plus-plus-test-objectives.md; docs/phase-1/mint-destroy-v1-development.md; BASE-06: docs/reviews/phase1-baseline/README.md; BASE-09: docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; docs/phase-1/W7-plus-plus-test-objectives.md; docs/phase-1/mint-destroy-v1-development.md; BASE-06: docs/reviews/phase1-baseline/README.md; BASE-09: docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N91" s="28" t="n"/>
@@ -7857,13 +7873,15 @@
       </c>
       <c r="I92" s="28" t="inlineStr">
         <is>
-          <t>Review 2026-10-28 (recorded evidence; no fresh acceptance run): Reviewed software and RTL reports explicitly exclude physical-board qualification. No new exact-build or board acceptance run was performed for this update.
+          <t>Update 2026-10-29 — combined candidate: Build IN PROGRESS as last reported: Vivado 2026.1 opened the validated checkpoint on 2026-10-29 at 18:13:31 (tool-reported time). No completed routing/timing/DRC result or combined BIT yet reported. No combined board programming. Earlier continuation-only BIT failed startup; that incident is not a physical result for the combined candidate.
+Earlier evidence: Review 2026-10-28 (recorded evidence; no fresh acceptance run): Reviewed software and RTL reports explicitly exclude physical-board qualification. No new exact-build or board acceptance run was performed for this update.
 Earlier baseline: No physical Phase 1 acceptance performed for this tracker.</t>
         </is>
       </c>
       <c r="J92" s="28" t="inlineStr">
         <is>
-          <t>After separate authorization, run H19/H20 with exact board/build identity and retained raw observations.
+          <t>Combined-candidate next action (2026-10-29): Obtain separate programming approval, temporarily load the exact reviewed BIT, then retain physical startup/recovery evidence; persistent flash stays unchanged.
+Original criterion / prior actions: After separate authorization, run H19/H20 with exact board/build identity and retained raw observations.
 Review action: Freeze the approved candidate and obtain matching build/timing/provenance plus separately authorized physical acceptance. Never relabel historical bitstreams.</t>
         </is>
       </c>
@@ -7874,12 +7892,12 @@
       </c>
       <c r="L92" s="28" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="M92" s="28" t="inlineStr">
         <is>
-          <t>docs/phase-1/W7-plus-plus-test-objectives.md; docs/phase-1/mint-destroy-v1-development.md; BASE-09: docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; docs/phase-1/W7-plus-plus-test-objectives.md; docs/phase-1/mint-destroy-v1-development.md; BASE-09: docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N92" s="28" t="n"/>
@@ -9025,12 +9043,14 @@
       </c>
       <c r="I110" s="28" t="inlineStr">
         <is>
-          <t>Unresolved fixture/implementation/oracle failures. Existing run: 8 failed, 46 passed. Failures cover SWITCH outcomes, delayed-fault issuer attribution, nested CALL/RETURN and saved-PC validation. No fresh RTL simulation was performed.</t>
+          <t>Update 2026-10-29 — combined candidate: Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery. Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0.
+Earlier evidence: Unresolved fixture/implementation/oracle failures. Existing run: 8 failed, 46 passed. Failures cover SWITCH outcomes, delayed-fault issuer attribution, nested CALL/RETURN and saved-PC validation. No fresh RTL simulation was performed.</t>
         </is>
       </c>
       <c r="J110" s="28" t="inlineStr">
         <is>
-          <t>Capture instruction words and pre-fault state, verify approved fixture encodings, then replay minimal isolated cases. Keep implementation defects possible until evidence excludes them.</t>
+          <t>Combined-candidate next action (2026-10-29): Retain earlier unrelated RTL failures as unresolved until individually rerun; this candidate does not close the whole regression suite.
+Original criterion / prior actions: Capture instruction words and pre-fault state, verify approved fixture encodings, then replay minimal isolated cases. Keep implementation defects possible until evidence excludes them.</t>
         </is>
       </c>
       <c r="K110" s="28" t="inlineStr">
@@ -9040,12 +9060,12 @@
       </c>
       <c r="L110" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="M110" s="28" t="inlineStr">
         <is>
-          <t>docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N110" s="28" t="n"/>
@@ -9078,7 +9098,7 @@
       </c>
       <c r="F111" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G111" s="28" t="inlineStr">
@@ -9093,12 +9113,14 @@
       </c>
       <c r="I111" s="28" t="inlineStr">
         <is>
-          <t>Reported generated-artifact/source mismatch; not freshly recomputed. Existing guard: RTLIL init ROM 2693 entries versus Python source 2694; 1 failed, 25 passed in that suite.</t>
+          <t>Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0.
+Earlier evidence: Reported generated-artifact/source mismatch; not freshly recomputed. Existing guard: RTLIL init ROM 2693 entries versus Python source 2694; 1 failed, 25 passed in that suite.</t>
         </is>
       </c>
       <c r="J111" s="28" t="inlineStr">
         <is>
-          <t>Freeze source and approved image first; then regenerate and qualify exact outputs under separate authorization. Do not equate a one-entry count fix with a qualified bitstream.</t>
+          <t>Combined-candidate next action (2026-10-29): Confirm combined initializer on the physical board after the routed build passes. Historical generator/count failures are not all closed by this isolated candidate.
+Original criterion / prior actions: Freeze source and approved image first; then regenerate and qualify exact outputs under separate authorization. Do not equate a one-entry count fix with a qualified bitstream.</t>
         </is>
       </c>
       <c r="K111" s="28" t="inlineStr">
@@ -9108,12 +9130,12 @@
       </c>
       <c r="L111" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="M111" s="28" t="inlineStr">
         <is>
-          <t>docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N111" s="28" t="n"/>
@@ -9284,7 +9306,7 @@
       </c>
       <c r="F114" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G114" s="28" t="inlineStr">
@@ -9299,12 +9321,14 @@
       </c>
       <c r="I114" s="28" t="inlineStr">
         <is>
-          <t>Confirmed current-source drift from recorded build. Fresh hash comparison finds 22 of 39 recorded input fingerprints differ from current files. The record's historical “verified” label is not qualification of today's source.</t>
+          <t>Update 2026-10-29 — combined candidate: Build IN PROGRESS as last reported: Vivado 2026.1 opened the validated checkpoint on 2026-10-29 at 18:13:31 (tool-reported time). No completed routing/timing/DRC result or combined BIT yet reported. No combined board programming.
+Earlier evidence: Confirmed current-source drift from recorded build. Fresh hash comparison finds 22 of 39 recorded input fingerprints differ from current files. The record's historical “verified” label is not qualification of today's source.</t>
         </is>
       </c>
       <c r="J114" s="28" t="inlineStr">
         <is>
-          <t>Freeze the candidate source/configuration; obtain matching generation, build/timing, artifact hashes and authorized physical evidence. Do not relabel the historical bitstream.</t>
+          <t>Combined-candidate next action (2026-10-29): Collect routed timing, DRC, output hashes and build receipt; historical source drift remains historical, not a reason to relabel old artifacts.
+Original criterion / prior actions: Freeze the candidate source/configuration; obtain matching generation, build/timing, artifact hashes and authorized physical evidence. Do not relabel the historical bitstream.</t>
         </is>
       </c>
       <c r="K114" s="28" t="inlineStr">
@@ -9314,12 +9338,12 @@
       </c>
       <c r="L114" s="28" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="M114" s="28" t="inlineStr">
         <is>
-          <t>docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; docs/reviews/phase1-baseline/README.md</t>
         </is>
       </c>
       <c r="N114" s="28" t="n"/>
@@ -9432,7 +9456,7 @@
       </c>
       <c r="B2" s="28" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C2" s="28" t="n"/>
@@ -9459,7 +9483,7 @@
       </c>
       <c r="B4" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Open")</f>
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -9485,7 +9509,7 @@
       </c>
       <c r="B6" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Not run")</f>
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C6" s="28" t="n"/>
       <c r="D6" s="28" t="n"/>
@@ -9498,7 +9522,7 @@
       </c>
       <c r="B7" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Needs verification")</f>
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C7" s="28" t="n"/>
       <c r="D7" s="28" t="n"/>
@@ -9972,7 +9996,7 @@
       </c>
       <c r="B7" s="28" t="inlineStr">
         <is>
-          <t>28 October update reviews recorded reports and prior-session focused tests; no fresh acceptance run. Threat Map, Summary and Method remain byte-for-byte unchanged. No W7 threat newly passed. Hardware, W7 baseline and full coverage remain separate gates.</t>
+          <t>29 October: user-supplied droplet logs and build preflight establish combined vendor boot and recovery-model passes. Implementation last reported in progress; combined physical acceptance not run. No W7 threat newly passed. Original threat sheets and historical criteria retained.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add W7 amoeba retry script and update test documentation and metadata
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
+++ b/docs/phase-1/CTMM_W7_Threat_Test_Plan.xlsx
@@ -11291,13 +11291,15 @@
       </c>
       <c r="I35" s="28" t="inlineStr">
         <is>
-          <t>Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0. Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery.
+          <t>Update 2026-10-30 — Amoeba retry: Exact-image frozen Amaranth RTL replay PASS: first intended Mallory fault, simulated manual reboot f, 1,854 post-reboot retirements across Boot/Alice/Mallory, retry branch, then the same intended Mallory fault. No root underflow. Frozen checksums unchanged. This is not a full vendor-mapped recovery replay. Bounded physical retry PASS: operator checksum-verified the exact BIT and supplied successful temporary-programming output for the recorded Wukong board. Startup plus six explicitly commanded manual reboots yielded seven complete CRC-valid fault snapshots, sequences 1 through 7. Each fault: code 8 at 0x3A08, Mallory CR12 0x0200000C. Every retry traversed 0x4638, not old root RETURN 0x463C. Alice advanced 42→43→44→45→46→47→48; no Boot/Alice fault or STACK_UNDERFLOW observed. Snapshot register/stack fields unchanged except sequence/CRC. This is stable exposed state, not an exhaustive stack-memory audit, indefinite recovery, automatic fault release, or live installed-image readback attestation.
+Earlier evidence: Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0. Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery.
 Earlier evidence: Defined objective; full acceptance not established by this tracker.</t>
         </is>
       </c>
       <c r="J35" s="28" t="inlineStr">
         <is>
-          <t>Combined-candidate next action (2026-10-29): Complete same-fixture cross-layer state comparison and separately authorized physical replay; boot-only vendor evidence does not establish mapped recovery.
+          <t>Amoeba retry next action (2026-10-30): Complete same-fixture behavioral/emitted/vendor-mapped/board committed-state comparisons. UART traces and fault snapshots are bounded observations, not complete memory equality.
+Original criterion / prior actions: Combined-candidate next action (2026-10-29): Complete same-fixture cross-layer state comparison and separately authorized physical replay; boot-only vendor evidence does not establish mapped recovery.
 Original criterion / prior actions: Compare committed registers/flags/memory/faults, not internal cycle counts except deadline/completion bounds. No forced X values or stale model accepted.</t>
         </is>
       </c>
@@ -11308,12 +11310,12 @@
       </c>
       <c r="L35" s="28" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="M35" s="28" t="inlineStr">
         <is>
-          <t>docs/phase-1/combined-validation-status-20261029.md; BASE-06: docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; BASE-06: docs/reviews/phase1-baseline/README.md; reports/amoeba-retry-candidate.md; generated-artifacts/amoeba-retry-preserved/vendor-verification.json; generated-artifacts/amoeba-retry-preserved/amoeba-retry-complete-evidence.zip</t>
         </is>
       </c>
       <c r="N35" s="28" t="n"/>
@@ -11361,13 +11363,15 @@
       </c>
       <c r="I36" s="28" t="inlineStr">
         <is>
-          <t>Update 2026-10-29 — combined candidate: Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery. Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0.
+          <t>Update 2026-10-30 — Amoeba retry: Bounded physical retry PASS: operator checksum-verified the exact BIT and supplied successful temporary-programming output for the recorded Wukong board. Startup plus six explicitly commanded manual reboots yielded seven complete CRC-valid fault snapshots, sequences 1 through 7. Each fault: code 8 at 0x3A08, Mallory CR12 0x0200000C. Every retry traversed 0x4638, not old root RETURN 0x463C. Alice advanced 42→43→44→45→46→47→48; no Boot/Alice fault or STACK_UNDERFLOW observed. Snapshot register/stack fields unchanged except sequence/CRC. This is stable exposed state, not an exhaustive stack-memory audit, indefinite recovery, automatic fault release, or live installed-image readback attestation.
+Earlier evidence: Update 2026-10-29 — combined candidate: Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery. Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0.
 Earlier evidence: Defined objective; full acceptance not established by this tracker.</t>
         </is>
       </c>
       <c r="J36" s="28" t="inlineStr">
         <is>
-          <t>Combined-candidate next action (2026-10-29): Perform exact combined-build cold/warm boots, repeated handoffs and physical recovery after separate programming approval.
+          <t>Amoeba retry next action (2026-10-30): Retain six successful manual retries; complete separately authorized cold/power-cycle and remaining retained-control/initialization objectives at the original scope.
+Original criterion / prior actions: Combined-candidate next action (2026-10-29): Perform exact combined-build cold/warm boots, repeated handoffs and physical recovery after separate programming approval.
 Original criterion / prior actions: Repeatable outcomes tied to bundle/input hashes, board identity, clock, logs and observed completion; no prior-run telemetry counted as new evidence.</t>
         </is>
       </c>
@@ -11378,12 +11382,12 @@
       </c>
       <c r="L36" s="28" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="M36" s="28" t="inlineStr">
         <is>
-          <t>docs/phase-1/combined-validation-status-20261029.md; BASE-06: docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; BASE-06: docs/reviews/phase1-baseline/README.md; reports/amoeba-retry-candidate.md; generated-artifacts/amoeba-retry-preserved/vendor-verification.json; generated-artifacts/amoeba-retry-preserved/amoeba-retry-complete-evidence.zip</t>
         </is>
       </c>
       <c r="N36" s="28" t="n"/>
@@ -12315,14 +12319,16 @@
       </c>
       <c r="I51" s="28" t="inlineStr">
         <is>
-          <t>Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0. Build IN PROGRESS as last reported: Vivado 2026.1 opened the validated checkpoint on 2026-10-29 at 18:13:31 (tool-reported time). No completed routing/timing/DRC result or combined BIT yet reported. No combined board programming.
+          <t>Update 2026-10-30 — Amoeba retry: Amoeba retry candidate build PASS: Vivado 2026.1, exit 0; setup +2.927 ns, hold +0.039 ns, pulse width +7.000 ns; zero reported timing failures. Uploaded vendor archive independently verified: 126 input hashes and 7 output hashes; manifest matches the locally prepared package. BIT SHA256 a4acb0ef9a39ba985d7769031cf146edb68fb65ff96e0b4f4a895093b54e5d4e; image SHA256 5603d8e105e47ca0f6524e4553989387c088de19ac0e6b3f6fd9897e170cf16d. No configuration-flash write or general production-release approval. Bounded physical retry PASS: operator checksum-verified the exact BIT and supplied successful temporary-programming output for the recorded Wukong board. Startup plus six explicitly commanded manual reboots yielded seven complete CRC-valid fault snapshots, sequences 1 through 7. Each fault: code 8 at 0x3A08, Mallory CR12 0x0200000C. Every retry traversed 0x4638, not old root RETURN 0x463C. Alice advanced 42→43→44→45→46→47→48; no Boot/Alice fault or STACK_UNDERFLOW observed. Snapshot register/stack fields unchanged except sequence/CRC. This is stable exposed state, not an exhaustive stack-memory audit, indefinite recovery, automatic fault release, or live installed-image readback attestation.
+Earlier evidence: Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0. Build IN PROGRESS as last reported: Vivado 2026.1 opened the validated checkpoint on 2026-10-29 at 18:13:31 (tool-reported time). No completed routing/timing/DRC result or combined BIT yet reported. No combined board programming.
 Earlier evidence: Review 2026-10-28 (recorded evidence; no fresh acceptance run): Saved actor report binds exact image/artifact identities. Named-CALL save reproduction rejects altered code and forged API metadata in isolated tests. This supports integrity/attribution, not full release or field coverage.
 Earlier baseline: Defined objective; full acceptance not established by this tracker.</t>
         </is>
       </c>
       <c r="J51" s="28" t="inlineStr">
         <is>
-          <t>Combined-candidate next action (2026-10-29): Retain image/source/checkpoint/evidence hashes, then bind the routed BIT receipt and physical observations; do not relabel the earlier BIT.
+          <t>Amoeba retry next action (2026-10-30): Exact BIT/image/build evidence is preserved for this candidate. Complete item-specific identity coverage and distinguish operator programming provenance from live data-image readback.
+Original criterion / prior actions: Combined-candidate next action (2026-10-29): Retain image/source/checkpoint/evidence hashes, then bind the routed BIT receipt and physical observations; do not relabel the earlier BIT.
 Original criterion / prior actions: Attach the actual LUMP/configuration and implementation identities to results; hardware claims identify the tested bitstream and board. Mark differences from simulator-only coverage.
 Review action: Complete item-specific identity/replay coverage and bind exact source, generated image, bitstream and physical observations.</t>
         </is>
@@ -12334,12 +12340,12 @@
       </c>
       <c r="L51" s="28" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="M51" s="28" t="inlineStr">
         <is>
-          <t>docs/phase-1/combined-validation-status-20261029.md; docs/reviews/saved-alice-mallory-execution.md; tests/server/test_named_call_save_attestation.py; BASE-09: docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; docs/reviews/saved-alice-mallory-execution.md; tests/server/test_named_call_save_attestation.py; BASE-09: docs/reviews/phase1-baseline/README.md; reports/amoeba-retry-candidate.md; generated-artifacts/amoeba-retry-preserved/vendor-verification.json; generated-artifacts/amoeba-retry-preserved/amoeba-retry-complete-evidence.zip</t>
         </is>
       </c>
       <c r="N51" s="28" t="n"/>
@@ -14683,13 +14689,15 @@
       <c r="H88" s="28" t="inlineStr"/>
       <c r="I88" s="28" t="inlineStr">
         <is>
-          <t>Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0. Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery.
+          <t>Update 2026-10-30 — Amoeba retry: Exact-image frozen Amaranth RTL replay PASS: first intended Mallory fault, simulated manual reboot f, 1,854 post-reboot retirements across Boot/Alice/Mallory, retry branch, then the same intended Mallory fault. No root underflow. Frozen checksums unchanged. This is not a full vendor-mapped recovery replay.
+Earlier evidence: Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0. Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery.
 Earlier evidence: Fresh combined verification: resident addresses 1024/7872, complete body identity, Thread ranges, matching Step-2 placements and private simulation checks pass without xfail exemptions. This is image-generator evidence only; same-byte simulator/RTL instruction conformance remains unverified.</t>
         </is>
       </c>
       <c r="J88" s="28" t="inlineStr">
         <is>
-          <t>Combined-candidate next action (2026-10-29): Retain this exact-image result without claiming full CHANGE/SWITCH or all-profile conformance.
+          <t>Amoeba retry next action (2026-10-30): Do not infer full CHANGE/SWITCH, Namespace geometry or all-profile conformance from this retry fixture.
+Original criterion / prior actions: Combined-candidate next action (2026-10-29): Retain this exact-image result without claiming full CHANGE/SWITCH or all-profile conformance.
 Original criterion / prior actions: Compare current ISA and simulator/RTL using immutable fixture identities and exact initial state.</t>
         </is>
       </c>
@@ -14700,12 +14708,12 @@
       </c>
       <c r="L88" s="28" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="M88" s="28" t="inlineStr">
         <is>
-          <t>docs/phase-1/combined-validation-status-20261029.md; BASE-04: docs/reviews/phase1-baseline/README.md; BASE-05: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md#combined-post-merge-verification--17-october-2026</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; BASE-04: docs/reviews/phase1-baseline/README.md; BASE-05: docs/reviews/phase1-baseline/README.md; docs/reviews/phase1-baseline/namespace-authority-progress.md#combined-post-merge-verification--17-october-2026; reports/amoeba-retry-candidate.md; generated-artifacts/amoeba-retry-preserved/vendor-verification.json; generated-artifacts/amoeba-retry-preserved/amoeba-retry-complete-evidence.zip</t>
         </is>
       </c>
       <c r="N88" s="28" t="n"/>
@@ -14749,13 +14757,15 @@
       <c r="H89" s="28" t="inlineStr"/>
       <c r="I89" s="28" t="inlineStr">
         <is>
-          <t>Update 2026-10-29 — combined candidate: Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery.
+          <t>Update 2026-10-30 — Amoeba retry: Exact-image frozen Amaranth RTL replay PASS: first intended Mallory fault, simulated manual reboot f, 1,854 post-reboot retirements across Boot/Alice/Mallory, retry branch, then the same intended Mallory fault. No root underflow. Frozen checksums unchanged. This is not a full vendor-mapped recovery replay. Bounded physical retry PASS: operator checksum-verified the exact BIT and supplied successful temporary-programming output for the recorded Wukong board. Startup plus six explicitly commanded manual reboots yielded seven complete CRC-valid fault snapshots, sequences 1 through 7. Each fault: code 8 at 0x3A08, Mallory CR12 0x0200000C. Every retry traversed 0x4638, not old root RETURN 0x463C. Alice advanced 42→43→44→45→46→47→48; no Boot/Alice fault or STACK_UNDERFLOW observed. Snapshot register/stack fields unchanged except sequence/CRC. This is stable exposed state, not an exhaustive stack-memory audit, indefinite recovery, automatic fault release, or live installed-image readback attestation.
+Earlier evidence: Update 2026-10-29 — combined candidate: Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery.
 Earlier evidence: Elapsed board clocks cannot be inferred from browser step speed.</t>
         </is>
       </c>
       <c r="J89" s="28" t="inlineStr">
         <is>
-          <t>Combined-candidate next action (2026-10-29): Verify remaining first-fault/precedence and physical timing objectives; model bounds are not FPGA elapsed-time measurements.
+          <t>Amoeba retry next action (2026-10-30): Keep remaining watchdog, competing-fault precedence and elapsed-time objectives open; manual f is not automatic fault authorization.
+Original criterion / prior actions: Combined-candidate next action (2026-10-29): Verify remaining first-fault/precedence and physical timing objectives; model bounds are not FPGA elapsed-time measurements.
 Original criterion / prior actions: Validate fault precedence and pre-recovery state; separate logical simulator checks from timed RTL/board proof.</t>
         </is>
       </c>
@@ -14766,12 +14776,12 @@
       </c>
       <c r="L89" s="28" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="M89" s="28" t="inlineStr">
         <is>
-          <t>docs/phase-1/combined-validation-status-20261029.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; reports/amoeba-retry-candidate.md; generated-artifacts/amoeba-retry-preserved/vendor-verification.json; generated-artifacts/amoeba-retry-preserved/amoeba-retry-complete-evidence.zip</t>
         </is>
       </c>
       <c r="N89" s="28" t="n"/>
@@ -14870,7 +14880,7 @@
       </c>
       <c r="F91" s="28" t="inlineStr">
         <is>
-          <t>Needs verification</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G91" s="28" t="inlineStr">
@@ -14881,14 +14891,16 @@
       <c r="H91" s="28" t="inlineStr"/>
       <c r="I91" s="28" t="inlineStr">
         <is>
-          <t>Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0. Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery. Build IN PROGRESS as last reported: Vivado 2026.1 opened the validated checkpoint on 2026-10-29 at 18:13:31 (tool-reported time). No completed routing/timing/DRC result or combined BIT yet reported. No combined board programming.
+          <t>Update 2026-10-30 — Amoeba retry: Amoeba retry candidate build PASS: Vivado 2026.1, exit 0; setup +2.927 ns, hold +0.039 ns, pulse width +7.000 ns; zero reported timing failures. Uploaded vendor archive independently verified: 126 input hashes and 7 output hashes; manifest matches the locally prepared package. BIT SHA256 a4acb0ef9a39ba985d7769031cf146edb68fb65ff96e0b4f4a895093b54e5d4e; image SHA256 5603d8e105e47ca0f6524e4553989387c088de19ac0e6b3f6fd9897e170cf16d. No configuration-flash write or general production-release approval.
+Earlier evidence: Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0. Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery. Build IN PROGRESS as last reported: Vivado 2026.1 opened the validated checkpoint on 2026-10-29 at 18:13:31 (tool-reported time). No completed routing/timing/DRC result or combined BIT yet reported. No combined board programming.
 Earlier evidence: Review 2026-10-28 (recorded evidence; no fresh acceptance run): Reviewed software and RTL reports explicitly exclude physical-board qualification. No new exact-build or board acceptance run was performed for this update.
 Earlier baseline: Prior inspection found 22/39 recorded build inputs differ; this is not a new build verification.</t>
         </is>
       </c>
       <c r="J91" s="28" t="inlineStr">
         <is>
-          <t>Combined-candidate next action (2026-10-29): Review COMBINED_IMPLEMENTATION_PASS, exit 0, timing/DRC reports and hash-bearing receipt before accepting the experimental build.
+          <t>Amoeba retry next action (2026-10-30): Exact candidate build-provenance criterion satisfied. Keep immutable history; broader release/physical gates remain separate.
+Original criterion / prior actions: Combined-candidate next action (2026-10-29): Review COMBINED_IMPLEMENTATION_PASS, exit 0, timing/DRC reports and hash-bearing receipt before accepting the experimental build.
 Original criterion / prior actions: Regenerate authorized exact inputs; verify hashes, ROM/configuration, timing, DRC and artifact sidecars.
 Review action: Freeze the approved candidate and obtain matching build/timing/provenance plus separately authorized physical acceptance. Never relabel historical bitstreams.</t>
         </is>
@@ -14900,12 +14912,12 @@
       </c>
       <c r="L91" s="28" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="M91" s="28" t="inlineStr">
         <is>
-          <t>docs/phase-1/combined-validation-status-20261029.md; docs/phase-1/W7-plus-plus-test-objectives.md; docs/phase-1/mint-destroy-v1-development.md; BASE-06: docs/reviews/phase1-baseline/README.md; BASE-09: docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; docs/phase-1/W7-plus-plus-test-objectives.md; docs/phase-1/mint-destroy-v1-development.md; BASE-06: docs/reviews/phase1-baseline/README.md; BASE-09: docs/reviews/phase1-baseline/README.md; reports/amoeba-retry-candidate.md; generated-artifacts/amoeba-retry-preserved/vendor-verification.json; generated-artifacts/amoeba-retry-preserved/amoeba-retry-complete-evidence.zip</t>
         </is>
       </c>
       <c r="N91" s="28" t="n"/>
@@ -14938,7 +14950,7 @@
       </c>
       <c r="F92" s="28" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="G92" s="28" t="inlineStr">
@@ -14953,14 +14965,16 @@
       </c>
       <c r="I92" s="28" t="inlineStr">
         <is>
-          <t>Update 2026-10-29 — combined candidate: Build IN PROGRESS as last reported: Vivado 2026.1 opened the validated checkpoint on 2026-10-29 at 18:13:31 (tool-reported time). No completed routing/timing/DRC result or combined BIT yet reported. No combined board programming. Earlier continuation-only BIT failed startup; that incident is not a physical result for the combined candidate.
+          <t>Update 2026-10-30 — Amoeba retry: Bounded physical retry PASS: operator checksum-verified the exact BIT and supplied successful temporary-programming output for the recorded Wukong board. Startup plus six explicitly commanded manual reboots yielded seven complete CRC-valid fault snapshots, sequences 1 through 7. Each fault: code 8 at 0x3A08, Mallory CR12 0x0200000C. Every retry traversed 0x4638, not old root RETURN 0x463C. Alice advanced 42→43→44→45→46→47→48; no Boot/Alice fault or STACK_UNDERFLOW observed. Snapshot register/stack fields unchanged except sequence/CRC. This is stable exposed state, not an exhaustive stack-memory audit, indefinite recovery, automatic fault release, or live installed-image readback attestation. Amoeba retry candidate build PASS: Vivado 2026.1, exit 0; setup +2.927 ns, hold +0.039 ns, pulse width +7.000 ns; zero reported timing failures. Uploaded vendor archive independently verified: 126 input hashes and 7 output hashes; manifest matches the locally prepared package. BIT SHA256 a4acb0ef9a39ba985d7769031cf146edb68fb65ff96e0b4f4a895093b54e5d4e; image SHA256 5603d8e105e47ca0f6524e4553989387c088de19ac0e6b3f6fd9897e170cf16d. No configuration-flash write or general production-release approval.
+Earlier evidence: Update 2026-10-29 — combined candidate: Build IN PROGRESS as last reported: Vivado 2026.1 opened the validated checkpoint on 2026-10-29 at 18:13:31 (tool-reported time). No completed routing/timing/DRC result or combined BIT yet reported. No combined board programming. Earlier continuation-only BIT failed startup; that incident is not a physical result for the combined candidate.
 Earlier evidence: Review 2026-10-28 (recorded evidence; no fresh acceptance run): Reviewed software and RTL reports explicitly exclude physical-board qualification. No new exact-build or board acceptance run was performed for this update.
 Earlier baseline: No physical Phase 1 acceptance performed for this tracker.</t>
         </is>
       </c>
       <c r="J92" s="28" t="inlineStr">
         <is>
-          <t>Combined-candidate next action (2026-10-29): Obtain separate programming approval, temporarily load the exact reviewed BIT, then retain physical startup/recovery evidence; persistent flash stays unchanged.
+          <t>Amoeba retry next action (2026-10-30): Bounded physical startup/retry passed. Complete remaining H19/H20 objectives before closing full physical acceptance; no flash approval.
+Original criterion / prior actions: Combined-candidate next action (2026-10-29): Obtain separate programming approval, temporarily load the exact reviewed BIT, then retain physical startup/recovery evidence; persistent flash stays unchanged.
 Original criterion / prior actions: After separate authorization, run H19/H20 with exact board/build identity and retained raw observations.
 Review action: Freeze the approved candidate and obtain matching build/timing/provenance plus separately authorized physical acceptance. Never relabel historical bitstreams.</t>
         </is>
@@ -14972,12 +14986,12 @@
       </c>
       <c r="L92" s="28" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="M92" s="28" t="inlineStr">
         <is>
-          <t>docs/phase-1/combined-validation-status-20261029.md; docs/phase-1/W7-plus-plus-test-objectives.md; docs/phase-1/mint-destroy-v1-development.md; BASE-09: docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; docs/phase-1/W7-plus-plus-test-objectives.md; docs/phase-1/mint-destroy-v1-development.md; BASE-09: docs/reviews/phase1-baseline/README.md; reports/amoeba-retry-candidate.md; generated-artifacts/amoeba-retry-preserved/vendor-verification.json; generated-artifacts/amoeba-retry-preserved/amoeba-retry-complete-evidence.zip</t>
         </is>
       </c>
       <c r="N92" s="28" t="n"/>
@@ -16123,13 +16137,15 @@
       </c>
       <c r="I110" s="28" t="inlineStr">
         <is>
-          <t>Update 2026-10-29 — combined candidate: Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery. Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0.
+          <t>Update 2026-10-30 — Amoeba retry: Exact-image frozen Amaranth RTL replay PASS: first intended Mallory fault, simulated manual reboot f, 1,854 post-reboot retirements across Boot/Alice/Mallory, retry branch, then the same intended Mallory fault. No root underflow. Frozen checksums unchanged. This is not a full vendor-mapped recovery replay. Bounded physical retry PASS: operator checksum-verified the exact BIT and supplied successful temporary-programming output for the recorded Wukong board. Startup plus six explicitly commanded manual reboots yielded seven complete CRC-valid fault snapshots, sequences 1 through 7. Each fault: code 8 at 0x3A08, Mallory CR12 0x0200000C. Every retry traversed 0x4638, not old root RETURN 0x463C. Alice advanced 42→43→44→45→46→47→48; no Boot/Alice fault or STACK_UNDERFLOW observed. Snapshot register/stack fields unchanged except sequence/CRC. This is stable exposed state, not an exhaustive stack-memory audit, indefinite recovery, automatic fault release, or live installed-image readback attestation.
+Earlier evidence: Update 2026-10-29 — combined candidate: Combined recovery-model PASS: model runner exit 0, subsequently accepted by the build preflight requiring the explicit pass marker and result JSON; one fault, authorized boot recovery, 100 post-recovery retirements, third address 0x2870. This is Amaranth simulated-UART evidence, not vendor-mapped recovery. Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0.
 Earlier evidence: Unresolved fixture/implementation/oracle failures. Existing run: 8 failed, 46 passed. Failures cover SWITCH outcomes, delayed-fault issuer attribution, nested CALL/RETURN and saved-PC validation. No fresh RTL simulation was performed.</t>
         </is>
       </c>
       <c r="J110" s="28" t="inlineStr">
         <is>
-          <t>Combined-candidate next action (2026-10-29): Retain earlier unrelated RTL failures as unresolved until individually rerun; this candidate does not close the whole regression suite.
+          <t>Amoeba retry next action (2026-10-30): Retain unrelated historical regression failures until individually rerun. This test does not close the whole RTL suite.
+Original criterion / prior actions: Combined-candidate next action (2026-10-29): Retain earlier unrelated RTL failures as unresolved until individually rerun; this candidate does not close the whole regression suite.
 Original criterion / prior actions: Capture instruction words and pre-fault state, verify approved fixture encodings, then replay minimal isolated cases. Keep implementation defects possible until evidence excludes them.</t>
         </is>
       </c>
@@ -16140,12 +16156,12 @@
       </c>
       <c r="L110" s="28" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="M110" s="28" t="inlineStr">
         <is>
-          <t>docs/phase-1/combined-validation-status-20261029.md; docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; docs/reviews/phase1-baseline/README.md; reports/amoeba-retry-candidate.md; generated-artifacts/amoeba-retry-preserved/vendor-verification.json; generated-artifacts/amoeba-retry-preserved/amoeba-retry-complete-evidence.zip</t>
         </is>
       </c>
       <c r="N110" s="28" t="n"/>
@@ -16193,13 +16209,15 @@
       </c>
       <c r="I111" s="28" t="inlineStr">
         <is>
-          <t>Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0.
+          <t>Update 2026-10-30 — Amoeba retry: Amoeba retry candidate build PASS: Vivado 2026.1, exit 0; setup +2.927 ns, hold +0.039 ns, pulse width +7.000 ns; zero reported timing failures. Uploaded vendor archive independently verified: 126 input hashes and 7 output hashes; manifest matches the locally prepared package. BIT SHA256 a4acb0ef9a39ba985d7769031cf146edb68fb65ff96e0b4f4a895093b54e5d4e; image SHA256 5603d8e105e47ca0f6524e4553989387c088de19ac0e6b3f6fd9897e170cf16d. No configuration-flash write or general production-release approval. Bounded physical retry PASS: operator checksum-verified the exact BIT and supplied successful temporary-programming output for the recorded Wukong board. Startup plus six explicitly commanded manual reboots yielded seven complete CRC-valid fault snapshots, sequences 1 through 7. Each fault: code 8 at 0x3A08, Mallory CR12 0x0200000C. Every retry traversed 0x4638, not old root RETURN 0x463C. Alice advanced 42→43→44→45→46→47→48; no Boot/Alice fault or STACK_UNDERFLOW observed. Snapshot register/stack fields unchanged except sequence/CRC. This is stable exposed state, not an exhaustive stack-memory audit, indefinite recovery, automatic fault release, or live installed-image readback attestation.
+Earlier evidence: Update 2026-10-29 — combined candidate: Combined frozen candidate: vendor-synthesized initialization/boot PASS; all 2,460 address/data writes checked, entry 0x4610 at 25 MHz. Original and corrected-observer checksums verified; vendor runner exit 0.
 Earlier evidence: Reported generated-artifact/source mismatch; not freshly recomputed. Existing guard: RTLIL init ROM 2693 entries versus Python source 2694; 1 failed, 25 passed in that suite.</t>
         </is>
       </c>
       <c r="J111" s="28" t="inlineStr">
         <is>
-          <t>Combined-candidate next action (2026-10-29): Confirm combined initializer on the physical board after the routed build passes. Historical generator/count failures are not all closed by this isolated candidate.
+          <t>Amoeba retry next action (2026-10-30): This candidate regenerated and booted physically. Retain broader generator/initializer and cold-start objectives until separately qualified.
+Original criterion / prior actions: Combined-candidate next action (2026-10-29): Confirm combined initializer on the physical board after the routed build passes. Historical generator/count failures are not all closed by this isolated candidate.
 Original criterion / prior actions: Freeze source and approved image first; then regenerate and qualify exact outputs under separate authorization. Do not equate a one-entry count fix with a qualified bitstream.</t>
         </is>
       </c>
@@ -16210,12 +16228,12 @@
       </c>
       <c r="L111" s="28" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="M111" s="28" t="inlineStr">
         <is>
-          <t>docs/phase-1/combined-validation-status-20261029.md; docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; docs/reviews/phase1-baseline/README.md; reports/amoeba-retry-candidate.md; generated-artifacts/amoeba-retry-preserved/vendor-verification.json; generated-artifacts/amoeba-retry-preserved/amoeba-retry-complete-evidence.zip</t>
         </is>
       </c>
       <c r="N111" s="28" t="n"/>
@@ -16386,7 +16404,7 @@
       </c>
       <c r="F114" s="28" t="inlineStr">
         <is>
-          <t>Needs verification</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G114" s="28" t="inlineStr">
@@ -16401,13 +16419,15 @@
       </c>
       <c r="I114" s="28" t="inlineStr">
         <is>
-          <t>Update 2026-10-29 — combined candidate: Build IN PROGRESS as last reported: Vivado 2026.1 opened the validated checkpoint on 2026-10-29 at 18:13:31 (tool-reported time). No completed routing/timing/DRC result or combined BIT yet reported. No combined board programming.
+          <t>Update 2026-10-30 — Amoeba retry: Amoeba retry candidate build PASS: Vivado 2026.1, exit 0; setup +2.927 ns, hold +0.039 ns, pulse width +7.000 ns; zero reported timing failures. Uploaded vendor archive independently verified: 126 input hashes and 7 output hashes; manifest matches the locally prepared package. BIT SHA256 a4acb0ef9a39ba985d7769031cf146edb68fb65ff96e0b4f4a895093b54e5d4e; image SHA256 5603d8e105e47ca0f6524e4553989387c088de19ac0e6b3f6fd9897e170cf16d. No configuration-flash write or general production-release approval.
+Earlier evidence: Update 2026-10-29 — combined candidate: Build IN PROGRESS as last reported: Vivado 2026.1 opened the validated checkpoint on 2026-10-29 at 18:13:31 (tool-reported time). No completed routing/timing/DRC result or combined BIT yet reported. No combined board programming.
 Earlier evidence: Confirmed current-source drift from recorded build. Fresh hash comparison finds 22 of 39 recorded input fingerprints differ from current files. The record's historical “verified” label is not qualification of today's source.</t>
         </is>
       </c>
       <c r="J114" s="28" t="inlineStr">
         <is>
-          <t>Combined-candidate next action (2026-10-29): Collect routed timing, DRC, output hashes and build receipt; historical source drift remains historical, not a reason to relabel old artifacts.
+          <t>Amoeba retry next action (2026-10-30): Exact candidate provenance gap closed; retain historical source-drift incidents without relabeling historical BITs.
+Original criterion / prior actions: Combined-candidate next action (2026-10-29): Collect routed timing, DRC, output hashes and build receipt; historical source drift remains historical, not a reason to relabel old artifacts.
 Original criterion / prior actions: Freeze the candidate source/configuration; obtain matching generation, build/timing, artifact hashes and authorized physical evidence. Do not relabel the historical bitstream.</t>
         </is>
       </c>
@@ -16418,12 +16438,12 @@
       </c>
       <c r="L114" s="28" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="M114" s="28" t="inlineStr">
         <is>
-          <t>docs/phase-1/combined-validation-status-20261029.md; docs/reviews/phase1-baseline/README.md</t>
+          <t>docs/phase-1/combined-validation-status-20261029.md; docs/reviews/phase1-baseline/README.md; reports/amoeba-retry-candidate.md; generated-artifacts/amoeba-retry-preserved/vendor-verification.json; generated-artifacts/amoeba-retry-preserved/amoeba-retry-complete-evidence.zip</t>
         </is>
       </c>
       <c r="N114" s="28" t="n"/>
@@ -16536,7 +16556,7 @@
       </c>
       <c r="B2" s="28" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C2" s="28" t="n"/>
@@ -16589,7 +16609,7 @@
       </c>
       <c r="B6" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Not run")</f>
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C6" s="28" t="n"/>
       <c r="D6" s="28" t="n"/>
@@ -16602,7 +16622,7 @@
       </c>
       <c r="B7" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Needs verification")</f>
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C7" s="28" t="n"/>
       <c r="D7" s="28" t="n"/>
@@ -16628,7 +16648,7 @@
       </c>
       <c r="B9" s="28">
         <f>COUNTIF(Completeness!F2:F10000,"Complete")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C9" s="28" t="n"/>
       <c r="D9" s="28" t="n"/>
@@ -16667,7 +16687,7 @@
       </c>
       <c r="B12" s="29">
         <f>IFERROR(COUNTIF(Completeness!F2:F10000,"Complete")/(COUNTA(Completeness!A2:A10000)-COUNTIF(Completeness!F2:F10000,"Out of scope")),0)</f>
-        <v>0.017857142857142856</v>
+        <v>0.03571428571428571</v>
       </c>
       <c r="C12" s="28" t="n"/>
       <c r="D12" s="28" t="n"/>
@@ -16853,7 +16873,7 @@
       </c>
       <c r="C22" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A22,Completeness!F2:F10000,"Complete")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A22,Completeness!F2:F10000,"Blocked")</f>
@@ -16967,7 +16987,7 @@
       </c>
       <c r="C28" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A28,Completeness!F2:F10000,"Complete")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28" s="28">
         <f>COUNTIFS(Completeness!B2:B10000,A28,Completeness!F2:F10000,"Blocked")</f>
@@ -17076,7 +17096,7 @@
       </c>
       <c r="B7" s="28" t="inlineStr">
         <is>
-          <t>29 October: user-supplied droplet logs and build preflight establish combined vendor boot and recovery-model passes. Implementation last reported in progress; combined physical acceptance not run. No W7 threat newly passed. Original threat sheets and historical criteria retained.</t>
+          <t>30 October: exact retry BIT build/provenance PASS, frozen Amaranth RTL retry PASS, physical startup and six manual retries PASS (snapshots 1–7; Alice 42→48; only intended Mallory faults). REL-01 and BASE-09 provenance complete. Full H19/H20 and REL-02 acceptance remains Needs verification; no new W7 threat closure, automatic recovery, flash programming or production-release approval. Original claims, scope baseline and historical evidence preserved.</t>
         </is>
       </c>
     </row>
@@ -18090,7 +18110,7 @@
       </c>
       <c r="B11" s="28" t="inlineStr">
         <is>
-          <t>Combined vendor boot and Amaranth recovery PASS only. Implementation last reported in progress. Combined physical acceptance pending; no new W7 closure.</t>
+          <t>30 October: exact retry BIT build/provenance PASS, frozen Amaranth RTL retry PASS, physical startup and six manual retries PASS (snapshots 1–7; Alice 42→48; only intended Mallory faults). REL-01 and BASE-09 provenance complete. Full H19/H20 and REL-02 acceptance remains Needs verification; no new W7 threat closure, automatic recovery, flash programming or production-release approval. Original claims, scope baseline and historical evidence preserved.</t>
         </is>
       </c>
     </row>

</xml_diff>